<commit_message>
auto: session 2026-08-05 10:55
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
+++ b/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
@@ -1256,7 +1256,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>booking trên báo tiền phong</t>
+          <t>booking quảng cáo thời báo kinh tế việt nam</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
@@ -1270,19 +1270,15 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Tiền Phong</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-tien-phong/</t>
-        </is>
-      </c>
+          <t>Thời báo Kinh tế Việt Nam (VnEconomy)</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>báo giá book bài pr trên vnexpress</t>
+          <t>booking trên báo tiền phong</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
@@ -1296,19 +1292,19 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>VnExpress</t>
+          <t>Tiền Phong</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>https://digicomvn.com/book-bao-vnexpress/</t>
+          <t>https://digicomvn.com/book-bao-tien-phong/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking afamily.vn</t>
+          <t>báo gia lai booking quảng cáo</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -1322,19 +1318,15 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Afamily</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-afamily/</t>
-        </is>
-      </c>
+          <t>Báo Gia Lai (báo tỉnh)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking bài pr admicro</t>
+          <t>báo giá book bài pr trên vnexpress</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
@@ -1348,15 +1340,19 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Admicro (Kênh14/CafeF network)</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr"/>
+          <t>VnExpress</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-vnexpress/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking báo công luận</t>
+          <t>báo giá booking afamily.vn</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -1370,15 +1366,19 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Công Luận</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr"/>
+          <t>Afamily</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-afamily/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking cafebiz</t>
+          <t>báo giá booking bài pr admicro</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
@@ -1392,19 +1392,15 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>CafeBiz</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-cafebiz/</t>
-        </is>
-      </c>
+          <t>Admicro (Kênh14/CafeF network)</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking chuyển động 24h</t>
+          <t>báo giá booking báo công luận</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
@@ -1418,19 +1414,15 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>24h</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-24h/</t>
-        </is>
-      </c>
+          <t>Công Luận</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking doanhnghiepphattrien</t>
+          <t>báo giá booking cafebiz</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
@@ -1444,15 +1436,19 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Doanh Nghiệp Phát Triển</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr"/>
+          <t>CafeBiz</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-cafebiz/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking doanhnghiepphattrien.vn</t>
+          <t>báo giá booking chuyển động 24h</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
@@ -1466,15 +1462,19 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Doanh Nghiệp Phát Triển</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr"/>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-24h/</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking kientrucvietnam.org</t>
+          <t>báo giá booking doanhnghiepphattrien</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Kiến Trúc Việt Nam</t>
+          <t>Doanh Nghiệp Phát Triển</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -1496,7 +1496,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking pr vnexpress</t>
+          <t>báo giá booking doanhnghiepphattrien.vn</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
@@ -1510,19 +1510,15 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>VnExpress</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-vnexpress/</t>
-        </is>
-      </c>
+          <t>Doanh Nghiệp Phát Triển</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking quảng cáo ione</t>
+          <t>báo giá booking kientrucvietnam.org</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
@@ -1536,7 +1532,7 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>iOne</t>
+          <t>Kiến Trúc Việt Nam</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -1544,7 +1540,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking quảng cáo ione.net</t>
+          <t>báo giá booking pr vnexpress</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
@@ -1558,15 +1554,19 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>iOne</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr"/>
+          <t>VnExpress</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-vnexpress/</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking saigon times</t>
+          <t>báo giá booking quảng cáo ione</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Saigon Times</t>
+          <t>iOne</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -1588,7 +1588,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking saigontime</t>
+          <t>báo giá booking quảng cáo ione.net</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Saigon Times</t>
+          <t>iOne</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr"/>
@@ -1610,7 +1610,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking saigontime quangcao</t>
+          <t>báo giá booking saigon times</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
@@ -1632,7 +1632,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking shoha.vn</t>
+          <t>báo giá booking saigontime</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
@@ -1646,19 +1646,15 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Soha (gõ nhầm shoha)</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-soha/</t>
-        </is>
-      </c>
+          <t>Saigon Times</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking soha.vn</t>
+          <t>báo giá booking saigontime quangcao</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
@@ -1672,19 +1668,15 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Soha</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-soha/</t>
-        </is>
-      </c>
+          <t>Saigon Times</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking thesaigontimes</t>
+          <t>báo giá booking shoha.vn</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
@@ -1698,15 +1690,19 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Saigon Times</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr"/>
+          <t>Soha (gõ nhầm shoha)</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-soha/</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking tuoitre.vn</t>
+          <t>báo giá booking soha.vn</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
@@ -1720,19 +1716,19 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Tuổi Trẻ</t>
+          <t>Soha</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
+          <t>https://digicomvn.com/book-bao-soha/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking tuổi trẻ</t>
+          <t>báo giá booking thesaigontimes</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
@@ -1746,19 +1742,15 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Tuổi Trẻ</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
-        </is>
-      </c>
+          <t>Saigon Times</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking vietnam news</t>
+          <t>báo giá booking tuoitre.vn</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
@@ -1772,15 +1764,19 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Vietnam News</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr"/>
+          <t>Tuổi Trẻ</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking vietnamnet</t>
+          <t>báo giá booking tuổi trẻ</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
@@ -1794,19 +1790,19 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>VietNamNet</t>
+          <t>Tuổi Trẻ</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>https://digicomvn.com/book-bao-vietnamnet/</t>
+          <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking vietnamnews</t>
+          <t>báo giá booking vietnam news</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
@@ -1828,7 +1824,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking vietnamnews.vn</t>
+          <t>báo giá booking vietnamnet</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
@@ -1842,15 +1838,19 @@
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Vietnam News</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr"/>
+          <t>VietNamNet</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-vietnamnet/</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>báo giá booking vnexpress 2019</t>
+          <t>báo giá booking vietnamnews</t>
         </is>
       </c>
       <c r="B58" s="4" t="n">
@@ -1864,19 +1864,15 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>VnExpress</t>
-        </is>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-vnexpress/</t>
-        </is>
-      </c>
+          <t>Vietnam News</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>bảng giá booking banner báo 24h</t>
+          <t>báo giá booking vietnamnews.vn</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
@@ -1890,19 +1886,15 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>24h</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-24h/</t>
-        </is>
-      </c>
+          <t>Vietnam News</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>bảng giá booking banner báo batdongsan.com.vn</t>
+          <t>báo giá booking vnexpress 2019</t>
         </is>
       </c>
       <c r="B60" s="4" t="n">
@@ -1916,15 +1908,19 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Batdongsan.com.vn</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr"/>
+          <t>VnExpress</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-vnexpress/</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>bảng giá booking banner báo nhipcaudautu</t>
+          <t>bảng giá booking banner báo 24h</t>
         </is>
       </c>
       <c r="B61" s="4" t="n">
@@ -1938,15 +1934,19 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Nhịp Cầu Đầu Tư</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr"/>
+          <t>24h</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-24h/</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>dịch vụ booking báo cafe f</t>
+          <t>bảng giá booking banner báo batdongsan.com.vn</t>
         </is>
       </c>
       <c r="B62" s="4" t="n">
@@ -1960,19 +1960,15 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>CafeF</t>
-        </is>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-cafef/</t>
-        </is>
-      </c>
+          <t>Batdongsan.com.vn</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>giá booking báo dep365</t>
+          <t>bảng giá booking banner báo nhipcaudautu</t>
         </is>
       </c>
       <c r="B63" s="4" t="n">
@@ -1986,7 +1982,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Đẹp365</t>
+          <t>Nhịp Cầu Đầu Tư</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr"/>
@@ -1994,7 +1990,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>giá booking báo heritage</t>
+          <t>dịch vụ booking báo cafe f</t>
         </is>
       </c>
       <c r="B64" s="4" t="n">
@@ -2008,15 +2004,19 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Heritage</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr"/>
+          <t>CafeF</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-cafef/</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>giá booking báo kiến trúc đời sống</t>
+          <t>giá booking báo dep365</t>
         </is>
       </c>
       <c r="B65" s="4" t="n">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Kiến Trúc Đời Sống</t>
+          <t>Đẹp365</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr"/>
@@ -2038,7 +2038,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>giá booking báo tuổi trẻ</t>
+          <t>giá booking báo heritage</t>
         </is>
       </c>
       <c r="B66" s="4" t="n">
@@ -2052,19 +2052,15 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Tuổi Trẻ</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
-        </is>
-      </c>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>kientrucvietnam.org.vn báo giá booking</t>
+          <t>giá booking báo kiến trúc đời sống</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
@@ -2078,61 +2074,71 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
+          <t>Kiến Trúc Đời Sống</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>giá booking báo tuổi trẻ</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Tuổi Trẻ</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>kientrucvietnam.org.vn báo giá booking</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
           <t>Kiến Trúc Việt Nam</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="inlineStr">
-        <is>
-          <t>booking quảng cáo báo</t>
-        </is>
-      </c>
-      <c r="B68" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="C68" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D68" s="6" t="inlineStr">
-        <is>
-          <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr"/>
-      <c r="F68" s="6" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>báo giá booking kols</t>
-        </is>
-      </c>
-      <c r="B69" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="C69" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="D69" s="6" t="inlineStr">
-        <is>
-          <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr"/>
-      <c r="F69" s="6" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>booking quảng cáo báo giấy</t>
+          <t>booking quảng cáo báo</t>
         </is>
       </c>
       <c r="B70" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C70" s="6" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>12</v>
+      </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
@@ -2144,13 +2150,15 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>booking quảng cáo báo mạng</t>
+          <t>báo giá booking kols</t>
         </is>
       </c>
       <c r="B71" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C71" s="6" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="C71" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
@@ -2162,7 +2170,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>báo giá booking banner web cafeland</t>
+          <t>booking quảng cáo báo giấy</t>
         </is>
       </c>
       <c r="B72" s="6" t="n">
@@ -2180,7 +2188,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>báo giá booking cpd banner homepage web cafeland</t>
+          <t>booking quảng cáo báo mạng</t>
         </is>
       </c>
       <c r="B73" s="6" t="n">
@@ -2198,7 +2206,7 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>báo giá booking fanpage</t>
+          <t>báo giá booking banner web cafeland</t>
         </is>
       </c>
       <c r="B74" s="6" t="n">
@@ -2216,7 +2224,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>báo giá booking kols 2019</t>
+          <t>báo giá booking cpd banner homepage web cafeland</t>
         </is>
       </c>
       <c r="B75" s="6" t="n">
@@ -2234,7 +2242,7 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>báo giá booking youtube</t>
+          <t>báo giá booking fanpage</t>
         </is>
       </c>
       <c r="B76" s="6" t="n">
@@ -2252,7 +2260,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>báo giá booking youtube channel</t>
+          <t>báo giá booking kols 2019</t>
         </is>
       </c>
       <c r="B77" s="6" t="n">
@@ -2270,7 +2278,7 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>bảng giá booking banner báo doanh nhân sài gofnn</t>
+          <t>báo giá booking quảng cáo</t>
         </is>
       </c>
       <c r="B78" s="6" t="n">
@@ -2288,7 +2296,7 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>bảng giá booking trên các fanpage báo chí</t>
+          <t>báo giá booking youtube</t>
         </is>
       </c>
       <c r="B79" s="6" t="n">
@@ -2304,81 +2312,81 @@
       <c r="F79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>chiến lược book bài báo chí</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C80" s="7" t="inlineStr"/>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>D. How-to / quy trình book báo</t>
-        </is>
-      </c>
-      <c r="E80" s="7" t="inlineStr"/>
-      <c r="F80" s="7" t="inlineStr"/>
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>báo giá booking youtube channel</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="6" t="inlineStr"/>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr"/>
+      <c r="F80" s="6" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="7" t="inlineStr">
-        <is>
-          <t>các bước book bài trên báo mạng</t>
-        </is>
-      </c>
-      <c r="B81" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C81" s="7" t="inlineStr"/>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>D. How-to / quy trình book báo</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="inlineStr"/>
-      <c r="F81" s="7" t="inlineStr"/>
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>bảng giá booking banner báo doanh nhân sài gofnn</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="6" t="inlineStr"/>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr"/>
+      <c r="F81" s="6" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="7" t="inlineStr">
-        <is>
-          <t>các tham số cần quan tam khi book báo marketing</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C82" s="7" t="inlineStr"/>
-      <c r="D82" s="7" t="inlineStr">
-        <is>
-          <t>D. How-to / quy trình book báo</t>
-        </is>
-      </c>
-      <c r="E82" s="7" t="inlineStr"/>
-      <c r="F82" s="7" t="inlineStr"/>
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>bảng giá booking trên các fanpage báo chí</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="6" t="inlineStr"/>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr"/>
+      <c r="F82" s="6" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>cách book bài pr trên báo chí</t>
-        </is>
-      </c>
-      <c r="B83" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C83" s="7" t="inlineStr"/>
-      <c r="D83" s="7" t="inlineStr">
-        <is>
-          <t>D. How-to / quy trình book báo</t>
-        </is>
-      </c>
-      <c r="E83" s="7" t="inlineStr"/>
-      <c r="F83" s="7" t="inlineStr"/>
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>các hình thức book bài quảng cáo trên các báo</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="6" t="inlineStr"/>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr"/>
+      <c r="F83" s="6" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>cách book bài trên báo mạng</t>
+          <t>chiến lược book bài báo chí</t>
         </is>
       </c>
       <c r="B84" s="7" t="n">
@@ -2396,7 +2404,7 @@
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>cách book bài viết trên báo mạng</t>
+          <t>các bước book bài trên báo mạng</t>
         </is>
       </c>
       <c r="B85" s="7" t="n">
@@ -2414,7 +2422,7 @@
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>cách book bài viết trên báo mạng bread and tea</t>
+          <t>các tham số cần quan tam khi book báo marketing</t>
         </is>
       </c>
       <c r="B86" s="7" t="n">
@@ -2432,7 +2440,7 @@
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>cách book bài viết trên báo mạng vietnambooking</t>
+          <t>cách book bài pr trên báo chí</t>
         </is>
       </c>
       <c r="B87" s="7" t="n">
@@ -2450,7 +2458,7 @@
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>hệ thống book bài pr trên các báo</t>
+          <t>cách book bài trên báo mạng</t>
         </is>
       </c>
       <c r="B88" s="7" t="n">
@@ -2466,85 +2474,85 @@
       <c r="F88" s="7" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t>agency booking báo chí</t>
-        </is>
-      </c>
-      <c r="B89" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="C89" s="8" t="inlineStr"/>
-      <c r="D89" s="8" t="inlineStr">
-        <is>
-          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
-        </is>
-      </c>
-      <c r="E89" s="8" t="inlineStr"/>
-      <c r="F89" s="8" t="inlineStr"/>
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>cách book bài viết trên báo mạng</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" s="7" t="inlineStr"/>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>D. How-to / quy trình book báo</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr"/>
+      <c r="F89" s="7" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="inlineStr">
-        <is>
-          <t>agency booking báo</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C90" s="8" t="inlineStr"/>
-      <c r="D90" s="8" t="inlineStr">
-        <is>
-          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
-        </is>
-      </c>
-      <c r="E90" s="8" t="inlineStr"/>
-      <c r="F90" s="8" t="inlineStr"/>
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>cách book bài viết trên báo mạng bread and tea</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="7" t="inlineStr"/>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>D. How-to / quy trình book báo</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr"/>
+      <c r="F90" s="7" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="inlineStr">
-        <is>
-          <t>agency book bài pr được các báo online nước ngoài</t>
-        </is>
-      </c>
-      <c r="B91" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C91" s="8" t="inlineStr"/>
-      <c r="D91" s="8" t="inlineStr">
-        <is>
-          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
-        </is>
-      </c>
-      <c r="E91" s="8" t="inlineStr"/>
-      <c r="F91" s="8" t="inlineStr"/>
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>cách book bài viết trên báo mạng vietnambooking</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C91" s="7" t="inlineStr"/>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>D. How-to / quy trình book báo</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr"/>
+      <c r="F91" s="7" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="inlineStr">
-        <is>
-          <t>công ty truyền thông booking báo mạng</t>
-        </is>
-      </c>
-      <c r="B92" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C92" s="8" t="inlineStr"/>
-      <c r="D92" s="8" t="inlineStr">
-        <is>
-          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
-        </is>
-      </c>
-      <c r="E92" s="8" t="inlineStr"/>
-      <c r="F92" s="8" t="inlineStr"/>
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>hệ thống book bài pr trên các báo</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" s="7" t="inlineStr"/>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>D. How-to / quy trình book báo</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr"/>
+      <c r="F92" s="7" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>dđơn vị chuyên nhận book báo</t>
+          <t>agency booking báo chí</t>
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C93" s="8" t="inlineStr"/>
       <c r="D93" s="8" t="inlineStr">
@@ -2558,11 +2566,11 @@
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>dđơn vị chuyên nhận book báo mycro</t>
+          <t>agency booking báo</t>
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C94" s="8" t="inlineStr"/>
       <c r="D94" s="8" t="inlineStr">
@@ -2576,7 +2584,7 @@
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>egency booking báo</t>
+          <t>agency book bài pr được các báo online nước ngoài</t>
         </is>
       </c>
       <c r="B95" s="8" t="n">
@@ -2594,7 +2602,7 @@
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>hoõ trợ booking báo mạng</t>
+          <t>công ty truyền thông booking báo mạng</t>
         </is>
       </c>
       <c r="B96" s="8" t="n">
@@ -2612,7 +2620,7 @@
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>hỗ trợ booking báo mạng</t>
+          <t>dđơn vị chuyên nhận book báo</t>
         </is>
       </c>
       <c r="B97" s="8" t="n">
@@ -2628,329 +2636,341 @@
       <c r="F97" s="8" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="9" t="inlineStr">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>dđơn vị chuyên nhận book báo mycro</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" s="8" t="inlineStr"/>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr"/>
+      <c r="F98" s="8" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>egency booking báo</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" s="8" t="inlineStr"/>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr"/>
+      <c r="F99" s="8" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>hoõ trợ booking báo mạng</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" s="8" t="inlineStr"/>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
+        </is>
+      </c>
+      <c r="E100" s="8" t="inlineStr"/>
+      <c r="F100" s="8" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>hỗ trợ booking báo mạng</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" s="8" t="inlineStr"/>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr"/>
+      <c r="F101" s="8" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>đơn vị nhận book bài viết báo at my</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C102" s="8" t="inlineStr"/>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
+        </is>
+      </c>
+      <c r="E102" s="8" t="inlineStr"/>
+      <c r="F102" s="8" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>báo giá booking báo đẹp</t>
         </is>
       </c>
-      <c r="B98" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C98" s="9" t="inlineStr"/>
-      <c r="D98" s="9" t="inlineStr">
+      <c r="B103" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" s="9" t="inlineStr"/>
+      <c r="D103" s="9" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E98" s="9" t="inlineStr"/>
-      <c r="F98" s="10" t="inlineStr">
+      <c r="E103" s="9" t="inlineStr"/>
+      <c r="F103" s="10" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="9" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="9" t="inlineStr">
         <is>
           <t>báo vlxd giá booking</t>
         </is>
       </c>
-      <c r="B99" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C99" s="9" t="inlineStr"/>
-      <c r="D99" s="9" t="inlineStr">
+      <c r="B104" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" s="9" t="inlineStr"/>
+      <c r="D104" s="9" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E99" s="9" t="inlineStr"/>
-      <c r="F99" s="10" t="inlineStr">
+      <c r="E104" s="9" t="inlineStr"/>
+      <c r="F104" s="10" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="9" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="9" t="inlineStr">
+        <is>
+          <t>bảng giá book bài các báo</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C105" s="9" t="inlineStr"/>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr"/>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/bang-gia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="inlineStr">
         <is>
           <t>bảng giá book báo tỉnh</t>
         </is>
       </c>
-      <c r="B100" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C100" s="9" t="inlineStr"/>
-      <c r="D100" s="9" t="inlineStr">
+      <c r="B106" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" s="9" t="inlineStr"/>
+      <c r="D106" s="9" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E100" s="9" t="inlineStr"/>
-      <c r="F100" s="10" t="inlineStr">
+      <c r="E106" s="9" t="inlineStr"/>
+      <c r="F106" s="10" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="11" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>tạp chí vật liệu xây dựng online báo giá booking</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C107" s="9" t="inlineStr"/>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr"/>
+      <c r="F107" s="10" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/bang-gia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="inlineStr">
         <is>
           <t>agency book bài pr trên báo cnn</t>
         </is>
       </c>
-      <c r="B101" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C101" s="11" t="inlineStr"/>
-      <c r="D101" s="11" t="inlineStr">
+      <c r="B108" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C108" s="11" t="inlineStr"/>
+      <c r="D108" s="11" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E101" s="11" t="inlineStr"/>
-      <c r="F101" s="12" t="inlineStr">
+      <c r="E108" s="11" t="inlineStr"/>
+      <c r="F108" s="12" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="11" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="11" t="inlineStr">
         <is>
           <t>agency book bài pr trên các báo nước ngoài</t>
         </is>
       </c>
-      <c r="B102" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C102" s="11" t="inlineStr"/>
-      <c r="D102" s="11" t="inlineStr">
+      <c r="B109" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" s="11" t="inlineStr"/>
+      <c r="D109" s="11" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E102" s="11" t="inlineStr"/>
-      <c r="F102" s="12" t="inlineStr">
+      <c r="E109" s="11" t="inlineStr"/>
+      <c r="F109" s="12" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="11" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="11" t="inlineStr">
         <is>
           <t>book bài pr trên báo nước ngoài cnn</t>
         </is>
       </c>
-      <c r="B103" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C103" s="11" t="inlineStr"/>
-      <c r="D103" s="11" t="inlineStr">
+      <c r="B110" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" s="11" t="inlineStr"/>
+      <c r="D110" s="11" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E103" s="11" t="inlineStr"/>
-      <c r="F103" s="12" t="inlineStr">
+      <c r="E110" s="11" t="inlineStr"/>
+      <c r="F110" s="12" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="11" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="11" t="inlineStr">
         <is>
           <t>book bài pr trên báo nước ngoài time</t>
         </is>
       </c>
-      <c r="B104" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C104" s="11" t="inlineStr"/>
-      <c r="D104" s="11" t="inlineStr">
+      <c r="B111" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C111" s="11" t="inlineStr"/>
+      <c r="D111" s="11" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E104" s="11" t="inlineStr"/>
-      <c r="F104" s="12" t="inlineStr">
+      <c r="E111" s="11" t="inlineStr"/>
+      <c r="F111" s="12" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="11" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="11" t="inlineStr">
         <is>
           <t>làm thế nào để booking online trên báo nước ngoài</t>
         </is>
       </c>
-      <c r="B105" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="11" t="inlineStr"/>
-      <c r="D105" s="11" t="inlineStr">
+      <c r="B112" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C112" s="11" t="inlineStr"/>
+      <c r="D112" s="11" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E105" s="11" t="inlineStr"/>
-      <c r="F105" s="12" t="inlineStr">
+      <c r="E112" s="11" t="inlineStr"/>
+      <c r="F112" s="12" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="13" t="inlineStr">
-        <is>
-          <t>book king báo mạng</t>
-        </is>
-      </c>
-      <c r="B106" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C106" s="13" t="inlineStr"/>
-      <c r="D106" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E106" s="13" t="inlineStr"/>
-      <c r="F106" s="13" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="13" t="inlineStr">
-        <is>
-          <t>book statement báo cáo kiểm tra sổ sách</t>
-        </is>
-      </c>
-      <c r="B107" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C107" s="13" t="inlineStr"/>
-      <c r="D107" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E107" s="13" t="inlineStr"/>
-      <c r="F107" s="13" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="13" t="inlineStr">
-        <is>
-          <t>book địa điểm trước khi họp báo</t>
-        </is>
-      </c>
-      <c r="B108" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C108" s="13" t="inlineStr"/>
-      <c r="D108" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E108" s="13" t="inlineStr"/>
-      <c r="F108" s="13" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="13" t="inlineStr">
-        <is>
-          <t>booking quảng cáo thời báo kinh tế việt nam</t>
-        </is>
-      </c>
-      <c r="B109" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C109" s="13" t="inlineStr"/>
-      <c r="D109" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E109" s="13" t="inlineStr"/>
-      <c r="F109" s="13" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="13" t="inlineStr">
-        <is>
-          <t>books trang tải báo</t>
-        </is>
-      </c>
-      <c r="B110" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C110" s="13" t="inlineStr"/>
-      <c r="D110" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E110" s="13" t="inlineStr"/>
-      <c r="F110" s="13" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="13" t="inlineStr">
-        <is>
-          <t>books.org trang tải báo</t>
-        </is>
-      </c>
-      <c r="B111" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C111" s="13" t="inlineStr"/>
-      <c r="D111" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E111" s="13" t="inlineStr"/>
-      <c r="F111" s="13" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="13" t="inlineStr">
-        <is>
-          <t>báo cáo kiểm tra sổ sách statement of books</t>
-        </is>
-      </c>
-      <c r="B112" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C112" s="13" t="inlineStr"/>
-      <c r="D112" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E112" s="13" t="inlineStr"/>
-      <c r="F112" s="13" t="inlineStr"/>
-    </row>
     <row r="113">
-      <c r="A113" s="13" t="inlineStr">
-        <is>
-          <t>báo cáo lỗi cho face book</t>
-        </is>
-      </c>
-      <c r="B113" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C113" s="13" t="inlineStr"/>
-      <c r="D113" s="13" t="inlineStr">
-        <is>
-          <t>Z. Rác - không liên quan</t>
-        </is>
-      </c>
-      <c r="E113" s="13" t="inlineStr"/>
-      <c r="F113" s="13" t="inlineStr"/>
+      <c r="A113" s="11" t="inlineStr">
+        <is>
+          <t>làm thế nào để booking online trên báo nước ngào</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" s="11" t="inlineStr"/>
+      <c r="D113" s="11" t="inlineStr">
+        <is>
+          <t>G. Booking báo quốc tế (CNN/Time...)</t>
+        </is>
+      </c>
+      <c r="E113" s="11" t="inlineStr"/>
+      <c r="F113" s="12" t="inlineStr">
+        <is>
+          <t>https://digicomvn.com/backlink-quoc-te/</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="13" t="inlineStr">
         <is>
-          <t>báo gia lai booking quảng cáo</t>
+          <t>book king báo mạng</t>
         </is>
       </c>
       <c r="B114" s="13" t="n">
@@ -2968,7 +2988,7 @@
     <row r="115">
       <c r="A115" s="13" t="inlineStr">
         <is>
-          <t>báo giá booking quảng cáo</t>
+          <t>book statement báo cáo kiểm tra sổ sách</t>
         </is>
       </c>
       <c r="B115" s="13" t="n">
@@ -2986,7 +3006,7 @@
     <row r="116">
       <c r="A116" s="13" t="inlineStr">
         <is>
-          <t>báo giá booking trang merry</t>
+          <t>book địa điểm trước khi họp báo</t>
         </is>
       </c>
       <c r="B116" s="13" t="n">
@@ -3004,7 +3024,7 @@
     <row r="117">
       <c r="A117" s="13" t="inlineStr">
         <is>
-          <t>báo giá life english book</t>
+          <t>books trang tải báo</t>
         </is>
       </c>
       <c r="B117" s="13" t="n">
@@ -3022,7 +3042,7 @@
     <row r="118">
       <c r="A118" s="13" t="inlineStr">
         <is>
-          <t>báo giá life english books</t>
+          <t>books.org trang tải báo</t>
         </is>
       </c>
       <c r="B118" s="13" t="n">
@@ -3040,7 +3060,7 @@
     <row r="119">
       <c r="A119" s="13" t="inlineStr">
         <is>
-          <t>báo giá surface pro book</t>
+          <t>báo cáo kiểm tra sổ sách statement of books</t>
         </is>
       </c>
       <c r="B119" s="13" t="n">
@@ -3058,7 +3078,7 @@
     <row r="120">
       <c r="A120" s="13" t="inlineStr">
         <is>
-          <t>bảng giá book bài các báo</t>
+          <t>báo cáo lỗi cho face book</t>
         </is>
       </c>
       <c r="B120" s="13" t="n">
@@ -3076,7 +3096,7 @@
     <row r="121">
       <c r="A121" s="13" t="inlineStr">
         <is>
-          <t>chặn thông báo face book đến mail</t>
+          <t>báo giá booking trang merry</t>
         </is>
       </c>
       <c r="B121" s="13" t="n">
@@ -3094,7 +3114,7 @@
     <row r="122">
       <c r="A122" s="13" t="inlineStr">
         <is>
-          <t>cài đặt tắt chuông báo face book</t>
+          <t>báo giá life english book</t>
         </is>
       </c>
       <c r="B122" s="13" t="n">
@@ -3112,7 +3132,7 @@
     <row r="123">
       <c r="A123" s="13" t="inlineStr">
         <is>
-          <t>các câu thông báo bán hàng trên face book</t>
+          <t>báo giá life english books</t>
         </is>
       </c>
       <c r="B123" s="13" t="n">
@@ -3130,7 +3150,7 @@
     <row r="124">
       <c r="A124" s="13" t="inlineStr">
         <is>
-          <t>các hình thức book bài quảng cáo trên các báo</t>
+          <t>báo giá surface pro book</t>
         </is>
       </c>
       <c r="B124" s="13" t="n">
@@ -3148,7 +3168,7 @@
     <row r="125">
       <c r="A125" s="13" t="inlineStr">
         <is>
-          <t>cách tắt thông báo sinh nhật cho face book</t>
+          <t>chặn thông báo face book đến mail</t>
         </is>
       </c>
       <c r="B125" s="13" t="n">
@@ -3166,7 +3186,7 @@
     <row r="126">
       <c r="A126" s="13" t="inlineStr">
         <is>
-          <t>email thông báo cho khách số booking khách sạn</t>
+          <t>cài đặt tắt chuông báo face book</t>
         </is>
       </c>
       <c r="B126" s="13" t="n">
@@ -3184,7 +3204,7 @@
     <row r="127">
       <c r="A127" s="13" t="inlineStr">
         <is>
-          <t>face book báo không thể thay đổi tên trang</t>
+          <t>các câu thông báo bán hàng trên face book</t>
         </is>
       </c>
       <c r="B127" s="13" t="n">
@@ -3202,7 +3222,7 @@
     <row r="128">
       <c r="A128" s="13" t="inlineStr">
         <is>
-          <t>face book báo lỗi vi phạm tiêu chuẩn cộng động</t>
+          <t>cách tắt thông báo sinh nhật cho face book</t>
         </is>
       </c>
       <c r="B128" s="13" t="n">
@@ -3220,7 +3240,7 @@
     <row r="129">
       <c r="A129" s="13" t="inlineStr">
         <is>
-          <t>face book báo something went wrong là bị gì</t>
+          <t>email thông báo cho khách số booking khách sạn</t>
         </is>
       </c>
       <c r="B129" s="13" t="n">
@@ -3238,7 +3258,7 @@
     <row r="130">
       <c r="A130" s="13" t="inlineStr">
         <is>
-          <t>face book báo đổi mật khẩu</t>
+          <t>face book báo không thể thay đổi tên trang</t>
         </is>
       </c>
       <c r="B130" s="13" t="n">
@@ -3256,7 +3276,7 @@
     <row r="131">
       <c r="A131" s="13" t="inlineStr">
         <is>
-          <t>face book bị báo cáo mạo danh</t>
+          <t>face book báo lỗi vi phạm tiêu chuẩn cộng động</t>
         </is>
       </c>
       <c r="B131" s="13" t="n">
@@ -3274,7 +3294,7 @@
     <row r="132">
       <c r="A132" s="13" t="inlineStr">
         <is>
-          <t>face book của nhà báo hoàng nguyên vũ</t>
+          <t>face book báo something went wrong là bị gì</t>
         </is>
       </c>
       <c r="B132" s="13" t="n">
@@ -3292,7 +3312,7 @@
     <row r="133">
       <c r="A133" s="13" t="inlineStr">
         <is>
-          <t>hiển thị thông báo của face book chrome</t>
+          <t>face book báo đổi mật khẩu</t>
         </is>
       </c>
       <c r="B133" s="13" t="n">
@@ -3310,7 +3330,7 @@
     <row r="134">
       <c r="A134" s="13" t="inlineStr">
         <is>
-          <t>huong dân xóa thông báo trên face book</t>
+          <t>face book bị báo cáo mạo danh</t>
         </is>
       </c>
       <c r="B134" s="13" t="n">
@@ -3328,7 +3348,7 @@
     <row r="135">
       <c r="A135" s="13" t="inlineStr">
         <is>
-          <t>hướng dẫn xóa thông báo trên face book</t>
+          <t>face book của nhà báo hoàng nguyên vũ</t>
         </is>
       </c>
       <c r="B135" s="13" t="n">
@@ -3346,7 +3366,7 @@
     <row r="136">
       <c r="A136" s="13" t="inlineStr">
         <is>
-          <t>không nhận thông báo mời chơi game từ face book</t>
+          <t>hiển thị thông báo của face book chrome</t>
         </is>
       </c>
       <c r="B136" s="13" t="n">
@@ -3364,7 +3384,7 @@
     <row r="137">
       <c r="A137" s="13" t="inlineStr">
         <is>
-          <t>không vào được face book báo lỗi proxy</t>
+          <t>huong dân xóa thông báo trên face book</t>
         </is>
       </c>
       <c r="B137" s="13" t="n">
@@ -3382,7 +3402,7 @@
     <row r="138">
       <c r="A138" s="13" t="inlineStr">
         <is>
-          <t>laàm sao biết ai báo cáo tên face book</t>
+          <t>hướng dẫn xóa thông báo trên face book</t>
         </is>
       </c>
       <c r="B138" s="13" t="n">
@@ -3400,7 +3420,7 @@
     <row r="139">
       <c r="A139" s="13" t="inlineStr">
         <is>
-          <t>làm thế nào để booking online trên báo nước ngào</t>
+          <t>không nhận thông báo mời chơi game từ face book</t>
         </is>
       </c>
       <c r="B139" s="13" t="n">
@@ -3418,7 +3438,7 @@
     <row r="140">
       <c r="A140" s="13" t="inlineStr">
         <is>
-          <t>my book live báo đèn đỏ</t>
+          <t>không vào được face book báo lỗi proxy</t>
         </is>
       </c>
       <c r="B140" s="13" t="n">
@@ -3436,7 +3456,7 @@
     <row r="141">
       <c r="A141" s="13" t="inlineStr">
         <is>
-          <t>nghiệp vụ báo giá và xác nhận booking note</t>
+          <t>laàm sao biết ai báo cáo tên face book</t>
         </is>
       </c>
       <c r="B141" s="13" t="n">
@@ -3454,7 +3474,7 @@
     <row r="142">
       <c r="A142" s="13" t="inlineStr">
         <is>
-          <t>statement of books báo cáo sổ sách</t>
+          <t>my book live báo đèn đỏ</t>
         </is>
       </c>
       <c r="B142" s="13" t="n">
@@ -3472,7 +3492,7 @@
     <row r="143">
       <c r="A143" s="13" t="inlineStr">
         <is>
-          <t>style book của tờ báo</t>
+          <t>nghiệp vụ báo giá và xác nhận booking note</t>
         </is>
       </c>
       <c r="B143" s="13" t="n">
@@ -3490,7 +3510,7 @@
     <row r="144">
       <c r="A144" s="13" t="inlineStr">
         <is>
-          <t>thoông báo khai trương face book the coffee house</t>
+          <t>statement of books báo cáo sổ sách</t>
         </is>
       </c>
       <c r="B144" s="13" t="n">
@@ -3508,7 +3528,7 @@
     <row r="145">
       <c r="A145" s="13" t="inlineStr">
         <is>
-          <t>thông báo khi booking trong wordpress</t>
+          <t>style book của tờ báo</t>
         </is>
       </c>
       <c r="B145" s="13" t="n">
@@ -3526,7 +3546,7 @@
     <row r="146">
       <c r="A146" s="13" t="inlineStr">
         <is>
-          <t>thông báo messenger khi book trong wordpress</t>
+          <t>thoông báo khai trương face book the coffee house</t>
         </is>
       </c>
       <c r="B146" s="13" t="n">
@@ -3544,7 +3564,7 @@
     <row r="147">
       <c r="A147" s="13" t="inlineStr">
         <is>
-          <t>thông báo thông báo khi book trong wordpress</t>
+          <t>thông báo khi booking trong wordpress</t>
         </is>
       </c>
       <c r="B147" s="13" t="n">
@@ -3562,7 +3582,7 @@
     <row r="148">
       <c r="A148" s="13" t="inlineStr">
         <is>
-          <t>thông báo về việc giao nhận booking trễ</t>
+          <t>thông báo messenger khi book trong wordpress</t>
         </is>
       </c>
       <c r="B148" s="13" t="n">
@@ -3580,7 +3600,7 @@
     <row r="149">
       <c r="A149" s="13" t="inlineStr">
         <is>
-          <t>thông báo đien lực đức thọ fa book hà tinh</t>
+          <t>thông báo thông báo khi book trong wordpress</t>
         </is>
       </c>
       <c r="B149" s="13" t="n">
@@ -3598,7 +3618,7 @@
     <row r="150">
       <c r="A150" s="13" t="inlineStr">
         <is>
-          <t>thông cáo báo chí thái hà books</t>
+          <t>thông báo về việc giao nhận booking trễ</t>
         </is>
       </c>
       <c r="B150" s="13" t="n">
@@ -3616,7 +3636,7 @@
     <row r="151">
       <c r="A151" s="13" t="inlineStr">
         <is>
-          <t>tạo tin báo trong face book</t>
+          <t>thông báo đien lực đức thọ fa book hà tinh</t>
         </is>
       </c>
       <c r="B151" s="13" t="n">
@@ -3634,7 +3654,7 @@
     <row r="152">
       <c r="A152" s="13" t="inlineStr">
         <is>
-          <t>tạp chí vật liệu xây dựng online báo giá booking</t>
+          <t>thông cáo báo chí thái hà books</t>
         </is>
       </c>
       <c r="B152" s="13" t="n">
@@ -3652,7 +3672,7 @@
     <row r="153">
       <c r="A153" s="13" t="inlineStr">
         <is>
-          <t>tắt thông báo bằng mail của booking và agoda</t>
+          <t>tạo tin báo trong face book</t>
         </is>
       </c>
       <c r="B153" s="13" t="n">
@@ -3670,7 +3690,7 @@
     <row r="154">
       <c r="A154" s="13" t="inlineStr">
         <is>
-          <t>tắt thông báo mini face book</t>
+          <t>tắt thông báo bằng mail của booking và agoda</t>
         </is>
       </c>
       <c r="B154" s="13" t="n">
@@ -3688,7 +3708,7 @@
     <row r="155">
       <c r="A155" s="13" t="inlineStr">
         <is>
-          <t>tắtht ông báo live strem và video trên face book</t>
+          <t>tắt thông báo mini face book</t>
         </is>
       </c>
       <c r="B155" s="13" t="n">
@@ -3706,7 +3726,7 @@
     <row r="156">
       <c r="A156" s="13" t="inlineStr">
         <is>
-          <t>vacpa e book báo cáo tài chính</t>
+          <t>tắtht ông báo live strem và video trên face book</t>
         </is>
       </c>
       <c r="B156" s="13" t="n">
@@ -3724,7 +3744,7 @@
     <row r="157">
       <c r="A157" s="13" t="inlineStr">
         <is>
-          <t>đơn vị nhận book bài viết báo at my</t>
+          <t>vacpa e book báo cáo tài chính</t>
         </is>
       </c>
       <c r="B157" s="13" t="n">
@@ -3767,29 +3787,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F110" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F111" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F113" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: session 2026-08-05 11:41
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
+++ b/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phan nhom tu khoa" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phan nhom tu khoa'!$A$1:$F$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Phan nhom tu khoa'!$A$1:$G$157</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -124,23 +124,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -506,15 +530,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F157"/>
+  <dimension ref="A1:G157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +573,11 @@
           <t>URL bài viết (đã có)</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Thực thể cần có (quét 15 đối thủ)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -572,6 +602,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -596,6 +631,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -620,6 +660,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -644,6 +689,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -666,6 +716,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -688,6 +743,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -710,6 +770,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -732,6 +797,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -754,6 +824,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -776,6 +851,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -798,6 +878,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -820,6 +905,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -842,6 +932,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -864,6 +959,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -886,6 +986,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -908,6 +1013,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -930,6 +1040,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -952,6 +1067,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -974,6 +1094,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -996,6 +1121,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1018,6 +1148,11 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1040,2727 +1175,3226 @@
           <t>https://digicomvn.com/booking-bao-pr/</t>
         </is>
       </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>booking báo vnexpress</t>
         </is>
       </c>
-      <c r="B24" s="4" t="n">
+      <c r="B24" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>VnExpress</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-vnexpress/</t>
         </is>
       </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>booking bài pr báo batdongsan.com.vn</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Batdongsan.com.vn</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>booking báo cafebiz</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>CafeBiz</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-cafebiz/</t>
         </is>
       </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>booking báo doanh nhân sài gòn cuối tuần</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Doanh Nhân Sài Gòn</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>booking báo dân trí</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Dân Trí</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-dan-tri/</t>
         </is>
       </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>booking báo forbes</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Forbes</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>booking báo phụ nữ online</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Phụ Nữ Online</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>booking báo sinh viên việt nam</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Sinh Viên Việt Nam</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr"/>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>booking quảng cáo báo nhịp cầu đầu tư</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Nhịp Cầu Đầu Tư</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>booking quảng cáo thời báo kinh tế việt nam</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Thời báo Kinh tế Việt Nam (VnEconomy)</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>booking trên báo tiền phong</t>
         </is>
       </c>
-      <c r="B34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Tiền Phong</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-tien-phong/</t>
         </is>
       </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>báo gia lai booking quảng cáo</t>
         </is>
       </c>
-      <c r="B35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>Báo Gia Lai (báo tỉnh)</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>báo giá book bài pr trên vnexpress</t>
         </is>
       </c>
-      <c r="B36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>VnExpress</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-vnexpress/</t>
         </is>
       </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>báo giá booking afamily.vn</t>
         </is>
       </c>
-      <c r="B37" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Afamily</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-afamily/</t>
         </is>
       </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>báo giá booking bài pr admicro</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>Admicro (Kênh14/CafeF network)</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>báo giá booking báo công luận</t>
         </is>
       </c>
-      <c r="B39" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>Công Luận</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>báo giá booking cafebiz</t>
         </is>
       </c>
-      <c r="B40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr"/>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>CafeBiz</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-cafebiz/</t>
         </is>
       </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>báo giá booking chuyển động 24h</t>
         </is>
       </c>
-      <c r="B41" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>24h</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-24h/</t>
         </is>
       </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>báo giá booking doanhnghiepphattrien</t>
         </is>
       </c>
-      <c r="B42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>Doanh Nghiệp Phát Triển</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>báo giá booking doanhnghiepphattrien.vn</t>
         </is>
       </c>
-      <c r="B43" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>Doanh Nghiệp Phát Triển</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>báo giá booking kientrucvietnam.org</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>Kiến Trúc Việt Nam</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>báo giá booking pr vnexpress</t>
         </is>
       </c>
-      <c r="B45" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>VnExpress</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-vnexpress/</t>
         </is>
       </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>báo giá booking quảng cáo ione</t>
         </is>
       </c>
-      <c r="B46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>iOne</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>báo giá booking quảng cáo ione.net</t>
         </is>
       </c>
-      <c r="B47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>iOne</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>báo giá booking saigon times</t>
         </is>
       </c>
-      <c r="B48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>Saigon Times</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>báo giá booking saigontime</t>
         </is>
       </c>
-      <c r="B49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Saigon Times</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>báo giá booking saigontime quangcao</t>
         </is>
       </c>
-      <c r="B50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="4" t="inlineStr"/>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>Saigon Times</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>báo giá booking shoha.vn</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C51" s="4" t="inlineStr"/>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Soha (gõ nhầm shoha)</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-soha/</t>
         </is>
       </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>báo giá booking soha.vn</t>
         </is>
       </c>
-      <c r="B52" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C52" s="4" t="inlineStr"/>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>Soha</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-soha/</t>
         </is>
       </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>báo giá booking thesaigontimes</t>
         </is>
       </c>
-      <c r="B53" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C53" s="4" t="inlineStr"/>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
         <is>
           <t>Saigon Times</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>báo giá booking tuoitre.vn</t>
         </is>
       </c>
-      <c r="B54" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C54" s="4" t="inlineStr"/>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>Tuổi Trẻ</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
         </is>
       </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>báo giá booking tuổi trẻ</t>
         </is>
       </c>
-      <c r="B55" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C55" s="4" t="inlineStr"/>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>Tuổi Trẻ</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
         </is>
       </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>báo giá booking vietnam news</t>
         </is>
       </c>
-      <c r="B56" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" s="4" t="inlineStr"/>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>Vietnam News</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr"/>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>báo giá booking vietnamnet</t>
         </is>
       </c>
-      <c r="B57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C57" s="4" t="inlineStr"/>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>VietNamNet</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-vietnamnet/</t>
         </is>
       </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>báo giá booking vietnamnews</t>
         </is>
       </c>
-      <c r="B58" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C58" s="4" t="inlineStr"/>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>Vietnam News</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr"/>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>báo giá booking vietnamnews.vn</t>
         </is>
       </c>
-      <c r="B59" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C59" s="4" t="inlineStr"/>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="B59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
         <is>
           <t>Vietnam News</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr"/>
+      <c r="F59" s="5" t="inlineStr"/>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>báo giá booking vnexpress 2019</t>
         </is>
       </c>
-      <c r="B60" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C60" s="4" t="inlineStr"/>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="B60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" s="5" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>VnExpress</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-vnexpress/</t>
         </is>
       </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>bảng giá booking banner báo 24h</t>
         </is>
       </c>
-      <c r="B61" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C61" s="4" t="inlineStr"/>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="B61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>24h</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-24h/</t>
         </is>
       </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>bảng giá booking banner báo batdongsan.com.vn</t>
         </is>
       </c>
-      <c r="B62" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C62" s="4" t="inlineStr"/>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="B62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>Batdongsan.com.vn</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>bảng giá booking banner báo nhipcaudautu</t>
         </is>
       </c>
-      <c r="B63" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C63" s="4" t="inlineStr"/>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="B63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>Nhịp Cầu Đầu Tư</t>
         </is>
       </c>
-      <c r="F63" s="4" t="inlineStr"/>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>dịch vụ booking báo cafe f</t>
         </is>
       </c>
-      <c r="B64" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C64" s="4" t="inlineStr"/>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="B64" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
         <is>
           <t>CafeF</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-cafef/</t>
         </is>
       </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>giá booking báo dep365</t>
         </is>
       </c>
-      <c r="B65" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C65" s="4" t="inlineStr"/>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="inlineStr">
+      <c r="B65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>Đẹp365</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr"/>
+      <c r="F65" s="5" t="inlineStr"/>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>giá booking báo heritage</t>
         </is>
       </c>
-      <c r="B66" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C66" s="4" t="inlineStr"/>
-      <c r="D66" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="B66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" s="5" t="inlineStr"/>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
         <is>
           <t>Heritage</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr"/>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="inlineStr">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>giá booking báo kiến trúc đời sống</t>
         </is>
       </c>
-      <c r="B67" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C67" s="4" t="inlineStr"/>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="B67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
         <is>
           <t>Kiến Trúc Đời Sống</t>
         </is>
       </c>
-      <c r="F67" s="4" t="inlineStr"/>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>giá booking báo tuổi trẻ</t>
         </is>
       </c>
-      <c r="B68" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C68" s="4" t="inlineStr"/>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="B68" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
         <is>
           <t>Tuổi Trẻ</t>
         </is>
       </c>
-      <c r="F68" s="5" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>https://digicomvn.com/book-bao-tuoi-tre/</t>
         </is>
       </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="inlineStr">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>kientrucvietnam.org.vn báo giá booking</t>
         </is>
       </c>
-      <c r="B69" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C69" s="4" t="inlineStr"/>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>B. Booking theo đầu báo cụ thể</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="B69" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>B. Booking theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
         <is>
           <t>Kiến Trúc Việt Nam</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr"/>
+      <c r="F69" s="5" t="inlineStr"/>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="inlineStr">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>booking quảng cáo báo</t>
         </is>
       </c>
-      <c r="B70" s="6" t="n">
+      <c r="B70" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="C70" s="6" t="n">
+      <c r="C70" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="D70" s="6" t="inlineStr">
+      <c r="D70" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E70" s="6" t="inlineStr"/>
-      <c r="F70" s="6" t="inlineStr"/>
+      <c r="E70" s="8" t="inlineStr"/>
+      <c r="F70" s="8" t="inlineStr"/>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <t>báo giá booking kols</t>
         </is>
       </c>
-      <c r="B71" s="6" t="n">
+      <c r="B71" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="C71" s="6" t="n">
+      <c r="C71" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="D71" s="6" t="inlineStr">
+      <c r="D71" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E71" s="6" t="inlineStr"/>
-      <c r="F71" s="6" t="inlineStr"/>
+      <c r="E71" s="8" t="inlineStr"/>
+      <c r="F71" s="8" t="inlineStr"/>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="inlineStr">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>booking quảng cáo báo giấy</t>
         </is>
       </c>
-      <c r="B72" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C72" s="6" t="inlineStr"/>
-      <c r="D72" s="6" t="inlineStr">
+      <c r="B72" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" s="8" t="inlineStr"/>
+      <c r="D72" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E72" s="6" t="inlineStr"/>
-      <c r="F72" s="6" t="inlineStr"/>
+      <c r="E72" s="8" t="inlineStr"/>
+      <c r="F72" s="8" t="inlineStr"/>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="inlineStr">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <t>booking quảng cáo báo mạng</t>
         </is>
       </c>
-      <c r="B73" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C73" s="6" t="inlineStr"/>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="B73" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73" s="8" t="inlineStr"/>
+      <c r="D73" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E73" s="6" t="inlineStr"/>
-      <c r="F73" s="6" t="inlineStr"/>
+      <c r="E73" s="8" t="inlineStr"/>
+      <c r="F73" s="8" t="inlineStr"/>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>báo giá booking banner web cafeland</t>
         </is>
       </c>
-      <c r="B74" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C74" s="6" t="inlineStr"/>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="B74" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="8" t="inlineStr"/>
+      <c r="D74" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr"/>
-      <c r="F74" s="6" t="inlineStr"/>
+      <c r="E74" s="8" t="inlineStr"/>
+      <c r="F74" s="8" t="inlineStr"/>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+      <c r="A75" s="8" t="inlineStr">
         <is>
           <t>báo giá booking cpd banner homepage web cafeland</t>
         </is>
       </c>
-      <c r="B75" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C75" s="6" t="inlineStr"/>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="B75" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" s="8" t="inlineStr"/>
+      <c r="D75" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E75" s="6" t="inlineStr"/>
-      <c r="F75" s="6" t="inlineStr"/>
+      <c r="E75" s="8" t="inlineStr"/>
+      <c r="F75" s="8" t="inlineStr"/>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>báo giá booking fanpage</t>
         </is>
       </c>
-      <c r="B76" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C76" s="6" t="inlineStr"/>
-      <c r="D76" s="6" t="inlineStr">
+      <c r="B76" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" s="8" t="inlineStr"/>
+      <c r="D76" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E76" s="6" t="inlineStr"/>
-      <c r="F76" s="6" t="inlineStr"/>
+      <c r="E76" s="8" t="inlineStr"/>
+      <c r="F76" s="8" t="inlineStr"/>
+      <c r="G76" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="inlineStr">
+      <c r="A77" s="8" t="inlineStr">
         <is>
           <t>báo giá booking kols 2019</t>
         </is>
       </c>
-      <c r="B77" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C77" s="6" t="inlineStr"/>
-      <c r="D77" s="6" t="inlineStr">
+      <c r="B77" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" s="8" t="inlineStr"/>
+      <c r="D77" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E77" s="6" t="inlineStr"/>
-      <c r="F77" s="6" t="inlineStr"/>
+      <c r="E77" s="8" t="inlineStr"/>
+      <c r="F77" s="8" t="inlineStr"/>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="inlineStr">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>báo giá booking quảng cáo</t>
         </is>
       </c>
-      <c r="B78" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C78" s="6" t="inlineStr"/>
-      <c r="D78" s="6" t="inlineStr">
+      <c r="B78" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" s="8" t="inlineStr"/>
+      <c r="D78" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr"/>
-      <c r="F78" s="6" t="inlineStr"/>
+      <c r="E78" s="8" t="inlineStr"/>
+      <c r="F78" s="8" t="inlineStr"/>
+      <c r="G78" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="inlineStr">
+      <c r="A79" s="8" t="inlineStr">
         <is>
           <t>báo giá booking youtube</t>
         </is>
       </c>
-      <c r="B79" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C79" s="6" t="inlineStr"/>
-      <c r="D79" s="6" t="inlineStr">
+      <c r="B79" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" s="8" t="inlineStr"/>
+      <c r="D79" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E79" s="6" t="inlineStr"/>
-      <c r="F79" s="6" t="inlineStr"/>
+      <c r="E79" s="8" t="inlineStr"/>
+      <c r="F79" s="8" t="inlineStr"/>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A80" s="8" t="inlineStr">
         <is>
           <t>báo giá booking youtube channel</t>
         </is>
       </c>
-      <c r="B80" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C80" s="6" t="inlineStr"/>
-      <c r="D80" s="6" t="inlineStr">
+      <c r="B80" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="8" t="inlineStr"/>
+      <c r="D80" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E80" s="6" t="inlineStr"/>
-      <c r="F80" s="6" t="inlineStr"/>
+      <c r="E80" s="8" t="inlineStr"/>
+      <c r="F80" s="8" t="inlineStr"/>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="inlineStr">
+      <c r="A81" s="8" t="inlineStr">
         <is>
           <t>bảng giá booking banner báo doanh nhân sài gofnn</t>
         </is>
       </c>
-      <c r="B81" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C81" s="6" t="inlineStr"/>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="B81" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="8" t="inlineStr"/>
+      <c r="D81" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E81" s="6" t="inlineStr"/>
-      <c r="F81" s="6" t="inlineStr"/>
+      <c r="E81" s="8" t="inlineStr"/>
+      <c r="F81" s="8" t="inlineStr"/>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
+      <c r="A82" s="8" t="inlineStr">
         <is>
           <t>bảng giá booking trên các fanpage báo chí</t>
         </is>
       </c>
-      <c r="B82" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C82" s="6" t="inlineStr"/>
-      <c r="D82" s="6" t="inlineStr">
+      <c r="B82" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="8" t="inlineStr"/>
+      <c r="D82" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr"/>
-      <c r="F82" s="6" t="inlineStr"/>
+      <c r="E82" s="8" t="inlineStr"/>
+      <c r="F82" s="8" t="inlineStr"/>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="inlineStr">
+      <c r="A83" s="8" t="inlineStr">
         <is>
           <t>các hình thức book bài quảng cáo trên các báo</t>
         </is>
       </c>
-      <c r="B83" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C83" s="6" t="inlineStr"/>
-      <c r="D83" s="6" t="inlineStr">
+      <c r="B83" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="8" t="inlineStr"/>
+      <c r="D83" s="8" t="inlineStr">
         <is>
           <t>C. Booking quảng cáo báo (banner/fanpage/youtube/KOLs)</t>
         </is>
       </c>
-      <c r="E83" s="6" t="inlineStr"/>
-      <c r="F83" s="6" t="inlineStr"/>
+      <c r="E83" s="8" t="inlineStr"/>
+      <c r="F83" s="8" t="inlineStr"/>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="7" t="inlineStr">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t>chiến lược book bài báo chí</t>
         </is>
       </c>
-      <c r="B84" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C84" s="7" t="inlineStr"/>
-      <c r="D84" s="7" t="inlineStr">
+      <c r="B84" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" s="10" t="inlineStr"/>
+      <c r="D84" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E84" s="7" t="inlineStr"/>
-      <c r="F84" s="7" t="inlineStr"/>
+      <c r="E84" s="10" t="inlineStr"/>
+      <c r="F84" s="10" t="inlineStr"/>
+      <c r="G84" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="7" t="inlineStr">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>các bước book bài trên báo mạng</t>
         </is>
       </c>
-      <c r="B85" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C85" s="7" t="inlineStr"/>
-      <c r="D85" s="7" t="inlineStr">
+      <c r="B85" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" s="10" t="inlineStr"/>
+      <c r="D85" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E85" s="7" t="inlineStr"/>
-      <c r="F85" s="7" t="inlineStr"/>
+      <c r="E85" s="10" t="inlineStr"/>
+      <c r="F85" s="10" t="inlineStr"/>
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="inlineStr">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>các tham số cần quan tam khi book báo marketing</t>
         </is>
       </c>
-      <c r="B86" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C86" s="7" t="inlineStr"/>
-      <c r="D86" s="7" t="inlineStr">
+      <c r="B86" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="10" t="inlineStr"/>
+      <c r="D86" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E86" s="7" t="inlineStr"/>
-      <c r="F86" s="7" t="inlineStr"/>
+      <c r="E86" s="10" t="inlineStr"/>
+      <c r="F86" s="10" t="inlineStr"/>
+      <c r="G86" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="7" t="inlineStr">
+      <c r="A87" s="10" t="inlineStr">
         <is>
           <t>cách book bài pr trên báo chí</t>
         </is>
       </c>
-      <c r="B87" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C87" s="7" t="inlineStr"/>
-      <c r="D87" s="7" t="inlineStr">
+      <c r="B87" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C87" s="10" t="inlineStr"/>
+      <c r="D87" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E87" s="7" t="inlineStr"/>
-      <c r="F87" s="7" t="inlineStr"/>
+      <c r="E87" s="10" t="inlineStr"/>
+      <c r="F87" s="10" t="inlineStr"/>
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="7" t="inlineStr">
+      <c r="A88" s="10" t="inlineStr">
         <is>
           <t>cách book bài trên báo mạng</t>
         </is>
       </c>
-      <c r="B88" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C88" s="7" t="inlineStr"/>
-      <c r="D88" s="7" t="inlineStr">
+      <c r="B88" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" s="10" t="inlineStr"/>
+      <c r="D88" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E88" s="7" t="inlineStr"/>
-      <c r="F88" s="7" t="inlineStr"/>
+      <c r="E88" s="10" t="inlineStr"/>
+      <c r="F88" s="10" t="inlineStr"/>
+      <c r="G88" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="7" t="inlineStr">
+      <c r="A89" s="10" t="inlineStr">
         <is>
           <t>cách book bài viết trên báo mạng</t>
         </is>
       </c>
-      <c r="B89" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C89" s="7" t="inlineStr"/>
-      <c r="D89" s="7" t="inlineStr">
+      <c r="B89" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" s="10" t="inlineStr"/>
+      <c r="D89" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E89" s="7" t="inlineStr"/>
-      <c r="F89" s="7" t="inlineStr"/>
+      <c r="E89" s="10" t="inlineStr"/>
+      <c r="F89" s="10" t="inlineStr"/>
+      <c r="G89" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="7" t="inlineStr">
+      <c r="A90" s="10" t="inlineStr">
         <is>
           <t>cách book bài viết trên báo mạng bread and tea</t>
         </is>
       </c>
-      <c r="B90" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C90" s="7" t="inlineStr"/>
-      <c r="D90" s="7" t="inlineStr">
+      <c r="B90" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="10" t="inlineStr"/>
+      <c r="D90" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E90" s="7" t="inlineStr"/>
-      <c r="F90" s="7" t="inlineStr"/>
+      <c r="E90" s="10" t="inlineStr"/>
+      <c r="F90" s="10" t="inlineStr"/>
+      <c r="G90" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="7" t="inlineStr">
+      <c r="A91" s="10" t="inlineStr">
         <is>
           <t>cách book bài viết trên báo mạng vietnambooking</t>
         </is>
       </c>
-      <c r="B91" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C91" s="7" t="inlineStr"/>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="B91" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C91" s="10" t="inlineStr"/>
+      <c r="D91" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E91" s="7" t="inlineStr"/>
-      <c r="F91" s="7" t="inlineStr"/>
+      <c r="E91" s="10" t="inlineStr"/>
+      <c r="F91" s="10" t="inlineStr"/>
+      <c r="G91" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="7" t="inlineStr">
+      <c r="A92" s="10" t="inlineStr">
         <is>
           <t>hệ thống book bài pr trên các báo</t>
         </is>
       </c>
-      <c r="B92" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C92" s="7" t="inlineStr"/>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="B92" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" s="10" t="inlineStr"/>
+      <c r="D92" s="10" t="inlineStr">
         <is>
           <t>D. How-to / quy trình book báo</t>
         </is>
       </c>
-      <c r="E92" s="7" t="inlineStr"/>
-      <c r="F92" s="7" t="inlineStr"/>
+      <c r="E92" s="10" t="inlineStr"/>
+      <c r="F92" s="10" t="inlineStr"/>
+      <c r="G92" s="11" t="inlineStr">
+        <is>
+          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="inlineStr">
+      <c r="A93" s="12" t="inlineStr">
         <is>
           <t>agency booking báo chí</t>
         </is>
       </c>
-      <c r="B93" s="8" t="n">
+      <c r="B93" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="C93" s="8" t="inlineStr"/>
-      <c r="D93" s="8" t="inlineStr">
+      <c r="C93" s="12" t="inlineStr"/>
+      <c r="D93" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E93" s="8" t="inlineStr"/>
-      <c r="F93" s="8" t="inlineStr"/>
+      <c r="E93" s="12" t="inlineStr"/>
+      <c r="F93" s="12" t="inlineStr"/>
+      <c r="G93" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+      <c r="A94" s="12" t="inlineStr">
         <is>
           <t>agency booking báo</t>
         </is>
       </c>
-      <c r="B94" s="8" t="n">
+      <c r="B94" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="C94" s="8" t="inlineStr"/>
-      <c r="D94" s="8" t="inlineStr">
+      <c r="C94" s="12" t="inlineStr"/>
+      <c r="D94" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E94" s="8" t="inlineStr"/>
-      <c r="F94" s="8" t="inlineStr"/>
+      <c r="E94" s="12" t="inlineStr"/>
+      <c r="F94" s="12" t="inlineStr"/>
+      <c r="G94" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="inlineStr">
+      <c r="A95" s="12" t="inlineStr">
         <is>
           <t>agency book bài pr được các báo online nước ngoài</t>
         </is>
       </c>
-      <c r="B95" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C95" s="8" t="inlineStr"/>
-      <c r="D95" s="8" t="inlineStr">
+      <c r="B95" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" s="12" t="inlineStr"/>
+      <c r="D95" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E95" s="8" t="inlineStr"/>
-      <c r="F95" s="8" t="inlineStr"/>
+      <c r="E95" s="12" t="inlineStr"/>
+      <c r="F95" s="12" t="inlineStr"/>
+      <c r="G95" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="inlineStr">
+      <c r="A96" s="12" t="inlineStr">
         <is>
           <t>công ty truyền thông booking báo mạng</t>
         </is>
       </c>
-      <c r="B96" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C96" s="8" t="inlineStr"/>
-      <c r="D96" s="8" t="inlineStr">
+      <c r="B96" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" s="12" t="inlineStr"/>
+      <c r="D96" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E96" s="8" t="inlineStr"/>
-      <c r="F96" s="8" t="inlineStr"/>
+      <c r="E96" s="12" t="inlineStr"/>
+      <c r="F96" s="12" t="inlineStr"/>
+      <c r="G96" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="inlineStr">
+      <c r="A97" s="12" t="inlineStr">
         <is>
           <t>dđơn vị chuyên nhận book báo</t>
         </is>
       </c>
-      <c r="B97" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C97" s="8" t="inlineStr"/>
-      <c r="D97" s="8" t="inlineStr">
+      <c r="B97" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" s="12" t="inlineStr"/>
+      <c r="D97" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E97" s="8" t="inlineStr"/>
-      <c r="F97" s="8" t="inlineStr"/>
+      <c r="E97" s="12" t="inlineStr"/>
+      <c r="F97" s="12" t="inlineStr"/>
+      <c r="G97" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="inlineStr">
+      <c r="A98" s="12" t="inlineStr">
         <is>
           <t>dđơn vị chuyên nhận book báo mycro</t>
         </is>
       </c>
-      <c r="B98" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C98" s="8" t="inlineStr"/>
-      <c r="D98" s="8" t="inlineStr">
+      <c r="B98" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" s="12" t="inlineStr"/>
+      <c r="D98" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E98" s="8" t="inlineStr"/>
-      <c r="F98" s="8" t="inlineStr"/>
+      <c r="E98" s="12" t="inlineStr"/>
+      <c r="F98" s="12" t="inlineStr"/>
+      <c r="G98" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
+      <c r="A99" s="12" t="inlineStr">
         <is>
           <t>egency booking báo</t>
         </is>
       </c>
-      <c r="B99" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C99" s="8" t="inlineStr"/>
-      <c r="D99" s="8" t="inlineStr">
+      <c r="B99" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" s="12" t="inlineStr"/>
+      <c r="D99" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E99" s="8" t="inlineStr"/>
-      <c r="F99" s="8" t="inlineStr"/>
+      <c r="E99" s="12" t="inlineStr"/>
+      <c r="F99" s="12" t="inlineStr"/>
+      <c r="G99" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
+      <c r="A100" s="12" t="inlineStr">
         <is>
           <t>hoõ trợ booking báo mạng</t>
         </is>
       </c>
-      <c r="B100" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C100" s="8" t="inlineStr"/>
-      <c r="D100" s="8" t="inlineStr">
+      <c r="B100" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" s="12" t="inlineStr"/>
+      <c r="D100" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E100" s="8" t="inlineStr"/>
-      <c r="F100" s="8" t="inlineStr"/>
+      <c r="E100" s="12" t="inlineStr"/>
+      <c r="F100" s="12" t="inlineStr"/>
+      <c r="G100" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
+      <c r="A101" s="12" t="inlineStr">
         <is>
           <t>hỗ trợ booking báo mạng</t>
         </is>
       </c>
-      <c r="B101" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C101" s="8" t="inlineStr"/>
-      <c r="D101" s="8" t="inlineStr">
+      <c r="B101" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" s="12" t="inlineStr"/>
+      <c r="D101" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E101" s="8" t="inlineStr"/>
-      <c r="F101" s="8" t="inlineStr"/>
+      <c r="E101" s="12" t="inlineStr"/>
+      <c r="F101" s="12" t="inlineStr"/>
+      <c r="G101" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="inlineStr">
+      <c r="A102" s="12" t="inlineStr">
         <is>
           <t>đơn vị nhận book bài viết báo at my</t>
         </is>
       </c>
-      <c r="B102" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C102" s="8" t="inlineStr"/>
-      <c r="D102" s="8" t="inlineStr">
+      <c r="B102" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C102" s="12" t="inlineStr"/>
+      <c r="D102" s="12" t="inlineStr">
         <is>
           <t>E. Agency/đơn vị booking báo (đối tượng bán dịch vụ B2B)</t>
         </is>
       </c>
-      <c r="E102" s="8" t="inlineStr"/>
-      <c r="F102" s="8" t="inlineStr"/>
+      <c r="E102" s="12" t="inlineStr"/>
+      <c r="F102" s="12" t="inlineStr"/>
+      <c r="G102" s="13" t="inlineStr">
+        <is>
+          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="9" t="inlineStr">
+      <c r="A103" s="14" t="inlineStr">
         <is>
           <t>báo giá booking báo đẹp</t>
         </is>
       </c>
-      <c r="B103" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C103" s="9" t="inlineStr"/>
-      <c r="D103" s="9" t="inlineStr">
+      <c r="B103" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C103" s="14" t="inlineStr"/>
+      <c r="D103" s="14" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E103" s="9" t="inlineStr"/>
-      <c r="F103" s="10" t="inlineStr">
+      <c r="E103" s="14" t="inlineStr"/>
+      <c r="F103" s="15" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
+      <c r="G103" s="16" t="inlineStr">
+        <is>
+          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="9" t="inlineStr">
+      <c r="A104" s="14" t="inlineStr">
         <is>
           <t>báo vlxd giá booking</t>
         </is>
       </c>
-      <c r="B104" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C104" s="9" t="inlineStr"/>
-      <c r="D104" s="9" t="inlineStr">
+      <c r="B104" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" s="14" t="inlineStr"/>
+      <c r="D104" s="14" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E104" s="9" t="inlineStr"/>
-      <c r="F104" s="10" t="inlineStr">
+      <c r="E104" s="14" t="inlineStr"/>
+      <c r="F104" s="15" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
+      <c r="G104" s="16" t="inlineStr">
+        <is>
+          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="9" t="inlineStr">
+      <c r="A105" s="14" t="inlineStr">
         <is>
           <t>bảng giá book bài các báo</t>
         </is>
       </c>
-      <c r="B105" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="9" t="inlineStr"/>
-      <c r="D105" s="9" t="inlineStr">
+      <c r="B105" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C105" s="14" t="inlineStr"/>
+      <c r="D105" s="14" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E105" s="9" t="inlineStr"/>
-      <c r="F105" s="10" t="inlineStr">
+      <c r="E105" s="14" t="inlineStr"/>
+      <c r="F105" s="15" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
+      <c r="G105" s="16" t="inlineStr">
+        <is>
+          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="9" t="inlineStr">
+      <c r="A106" s="14" t="inlineStr">
         <is>
           <t>bảng giá book báo tỉnh</t>
         </is>
       </c>
-      <c r="B106" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C106" s="9" t="inlineStr"/>
-      <c r="D106" s="9" t="inlineStr">
+      <c r="B106" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" s="14" t="inlineStr"/>
+      <c r="D106" s="14" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E106" s="9" t="inlineStr"/>
-      <c r="F106" s="10" t="inlineStr">
+      <c r="E106" s="14" t="inlineStr"/>
+      <c r="F106" s="15" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
+      <c r="G106" s="16" t="inlineStr">
+        <is>
+          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="9" t="inlineStr">
+      <c r="A107" s="14" t="inlineStr">
         <is>
           <t>tạp chí vật liệu xây dựng online báo giá booking</t>
         </is>
       </c>
-      <c r="B107" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C107" s="9" t="inlineStr"/>
-      <c r="D107" s="9" t="inlineStr">
+      <c r="B107" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C107" s="14" t="inlineStr"/>
+      <c r="D107" s="14" t="inlineStr">
         <is>
           <t>F. Báo giá booking báo (chung, không rõ đầu báo)</t>
         </is>
       </c>
-      <c r="E107" s="9" t="inlineStr"/>
-      <c r="F107" s="10" t="inlineStr">
+      <c r="E107" s="14" t="inlineStr"/>
+      <c r="F107" s="15" t="inlineStr">
         <is>
           <t>https://digicomvn.com/bang-gia/</t>
         </is>
       </c>
+      <c r="G107" s="16" t="inlineStr">
+        <is>
+          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="11" t="inlineStr">
+      <c r="A108" s="17" t="inlineStr">
         <is>
           <t>agency book bài pr trên báo cnn</t>
         </is>
       </c>
-      <c r="B108" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C108" s="11" t="inlineStr"/>
-      <c r="D108" s="11" t="inlineStr">
+      <c r="B108" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C108" s="17" t="inlineStr"/>
+      <c r="D108" s="17" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E108" s="11" t="inlineStr"/>
-      <c r="F108" s="12" t="inlineStr">
+      <c r="E108" s="17" t="inlineStr"/>
+      <c r="F108" s="18" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
+      <c r="G108" s="19" t="inlineStr">
+        <is>
+          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="11" t="inlineStr">
+      <c r="A109" s="17" t="inlineStr">
         <is>
           <t>agency book bài pr trên các báo nước ngoài</t>
         </is>
       </c>
-      <c r="B109" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C109" s="11" t="inlineStr"/>
-      <c r="D109" s="11" t="inlineStr">
+      <c r="B109" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" s="17" t="inlineStr"/>
+      <c r="D109" s="17" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E109" s="11" t="inlineStr"/>
-      <c r="F109" s="12" t="inlineStr">
+      <c r="E109" s="17" t="inlineStr"/>
+      <c r="F109" s="18" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
+      <c r="G109" s="19" t="inlineStr">
+        <is>
+          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="11" t="inlineStr">
+      <c r="A110" s="17" t="inlineStr">
         <is>
           <t>book bài pr trên báo nước ngoài cnn</t>
         </is>
       </c>
-      <c r="B110" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C110" s="11" t="inlineStr"/>
-      <c r="D110" s="11" t="inlineStr">
+      <c r="B110" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" s="17" t="inlineStr"/>
+      <c r="D110" s="17" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E110" s="11" t="inlineStr"/>
-      <c r="F110" s="12" t="inlineStr">
+      <c r="E110" s="17" t="inlineStr"/>
+      <c r="F110" s="18" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
+      <c r="G110" s="19" t="inlineStr">
+        <is>
+          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="11" t="inlineStr">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>book bài pr trên báo nước ngoài time</t>
         </is>
       </c>
-      <c r="B111" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C111" s="11" t="inlineStr"/>
-      <c r="D111" s="11" t="inlineStr">
+      <c r="B111" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C111" s="17" t="inlineStr"/>
+      <c r="D111" s="17" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E111" s="11" t="inlineStr"/>
-      <c r="F111" s="12" t="inlineStr">
+      <c r="E111" s="17" t="inlineStr"/>
+      <c r="F111" s="18" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
+      <c r="G111" s="19" t="inlineStr">
+        <is>
+          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+        </is>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="11" t="inlineStr">
+      <c r="A112" s="17" t="inlineStr">
         <is>
           <t>làm thế nào để booking online trên báo nước ngoài</t>
         </is>
       </c>
-      <c r="B112" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C112" s="11" t="inlineStr"/>
-      <c r="D112" s="11" t="inlineStr">
+      <c r="B112" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C112" s="17" t="inlineStr"/>
+      <c r="D112" s="17" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E112" s="11" t="inlineStr"/>
-      <c r="F112" s="12" t="inlineStr">
+      <c r="E112" s="17" t="inlineStr"/>
+      <c r="F112" s="18" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
+      <c r="G112" s="19" t="inlineStr">
+        <is>
+          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+        </is>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="11" t="inlineStr">
+      <c r="A113" s="17" t="inlineStr">
         <is>
           <t>làm thế nào để booking online trên báo nước ngào</t>
         </is>
       </c>
-      <c r="B113" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C113" s="11" t="inlineStr"/>
-      <c r="D113" s="11" t="inlineStr">
+      <c r="B113" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" s="17" t="inlineStr"/>
+      <c r="D113" s="17" t="inlineStr">
         <is>
           <t>G. Booking báo quốc tế (CNN/Time...)</t>
         </is>
       </c>
-      <c r="E113" s="11" t="inlineStr"/>
-      <c r="F113" s="12" t="inlineStr">
+      <c r="E113" s="17" t="inlineStr"/>
+      <c r="F113" s="18" t="inlineStr">
         <is>
           <t>https://digicomvn.com/backlink-quoc-te/</t>
         </is>
       </c>
+      <c r="G113" s="19" t="inlineStr">
+        <is>
+          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="13" t="inlineStr">
+      <c r="A114" s="20" t="inlineStr">
         <is>
           <t>book king báo mạng</t>
         </is>
       </c>
-      <c r="B114" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C114" s="13" t="inlineStr"/>
-      <c r="D114" s="13" t="inlineStr">
+      <c r="B114" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C114" s="20" t="inlineStr"/>
+      <c r="D114" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E114" s="13" t="inlineStr"/>
-      <c r="F114" s="13" t="inlineStr"/>
+      <c r="E114" s="20" t="inlineStr"/>
+      <c r="F114" s="20" t="inlineStr"/>
+      <c r="G114" s="21" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="13" t="inlineStr">
+      <c r="A115" s="20" t="inlineStr">
         <is>
           <t>book statement báo cáo kiểm tra sổ sách</t>
         </is>
       </c>
-      <c r="B115" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C115" s="13" t="inlineStr"/>
-      <c r="D115" s="13" t="inlineStr">
+      <c r="B115" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C115" s="20" t="inlineStr"/>
+      <c r="D115" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E115" s="13" t="inlineStr"/>
-      <c r="F115" s="13" t="inlineStr"/>
+      <c r="E115" s="20" t="inlineStr"/>
+      <c r="F115" s="20" t="inlineStr"/>
+      <c r="G115" s="21" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" s="13" t="inlineStr">
+      <c r="A116" s="20" t="inlineStr">
         <is>
           <t>book địa điểm trước khi họp báo</t>
         </is>
       </c>
-      <c r="B116" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C116" s="13" t="inlineStr"/>
-      <c r="D116" s="13" t="inlineStr">
+      <c r="B116" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C116" s="20" t="inlineStr"/>
+      <c r="D116" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E116" s="13" t="inlineStr"/>
-      <c r="F116" s="13" t="inlineStr"/>
+      <c r="E116" s="20" t="inlineStr"/>
+      <c r="F116" s="20" t="inlineStr"/>
+      <c r="G116" s="21" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" s="13" t="inlineStr">
+      <c r="A117" s="20" t="inlineStr">
         <is>
           <t>books trang tải báo</t>
         </is>
       </c>
-      <c r="B117" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C117" s="13" t="inlineStr"/>
-      <c r="D117" s="13" t="inlineStr">
+      <c r="B117" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C117" s="20" t="inlineStr"/>
+      <c r="D117" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E117" s="13" t="inlineStr"/>
-      <c r="F117" s="13" t="inlineStr"/>
+      <c r="E117" s="20" t="inlineStr"/>
+      <c r="F117" s="20" t="inlineStr"/>
+      <c r="G117" s="21" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" s="13" t="inlineStr">
+      <c r="A118" s="20" t="inlineStr">
         <is>
           <t>books.org trang tải báo</t>
         </is>
       </c>
-      <c r="B118" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C118" s="13" t="inlineStr"/>
-      <c r="D118" s="13" t="inlineStr">
+      <c r="B118" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C118" s="20" t="inlineStr"/>
+      <c r="D118" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E118" s="13" t="inlineStr"/>
-      <c r="F118" s="13" t="inlineStr"/>
+      <c r="E118" s="20" t="inlineStr"/>
+      <c r="F118" s="20" t="inlineStr"/>
+      <c r="G118" s="21" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" s="13" t="inlineStr">
+      <c r="A119" s="20" t="inlineStr">
         <is>
           <t>báo cáo kiểm tra sổ sách statement of books</t>
         </is>
       </c>
-      <c r="B119" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C119" s="13" t="inlineStr"/>
-      <c r="D119" s="13" t="inlineStr">
+      <c r="B119" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C119" s="20" t="inlineStr"/>
+      <c r="D119" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E119" s="13" t="inlineStr"/>
-      <c r="F119" s="13" t="inlineStr"/>
+      <c r="E119" s="20" t="inlineStr"/>
+      <c r="F119" s="20" t="inlineStr"/>
+      <c r="G119" s="21" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="13" t="inlineStr">
+      <c r="A120" s="20" t="inlineStr">
         <is>
           <t>báo cáo lỗi cho face book</t>
         </is>
       </c>
-      <c r="B120" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C120" s="13" t="inlineStr"/>
-      <c r="D120" s="13" t="inlineStr">
+      <c r="B120" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C120" s="20" t="inlineStr"/>
+      <c r="D120" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E120" s="13" t="inlineStr"/>
-      <c r="F120" s="13" t="inlineStr"/>
+      <c r="E120" s="20" t="inlineStr"/>
+      <c r="F120" s="20" t="inlineStr"/>
+      <c r="G120" s="21" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" s="13" t="inlineStr">
+      <c r="A121" s="20" t="inlineStr">
         <is>
           <t>báo giá booking trang merry</t>
         </is>
       </c>
-      <c r="B121" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C121" s="13" t="inlineStr"/>
-      <c r="D121" s="13" t="inlineStr">
+      <c r="B121" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C121" s="20" t="inlineStr"/>
+      <c r="D121" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E121" s="13" t="inlineStr"/>
-      <c r="F121" s="13" t="inlineStr"/>
+      <c r="E121" s="20" t="inlineStr"/>
+      <c r="F121" s="20" t="inlineStr"/>
+      <c r="G121" s="21" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="13" t="inlineStr">
+      <c r="A122" s="20" t="inlineStr">
         <is>
           <t>báo giá life english book</t>
         </is>
       </c>
-      <c r="B122" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C122" s="13" t="inlineStr"/>
-      <c r="D122" s="13" t="inlineStr">
+      <c r="B122" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C122" s="20" t="inlineStr"/>
+      <c r="D122" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E122" s="13" t="inlineStr"/>
-      <c r="F122" s="13" t="inlineStr"/>
+      <c r="E122" s="20" t="inlineStr"/>
+      <c r="F122" s="20" t="inlineStr"/>
+      <c r="G122" s="21" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" s="13" t="inlineStr">
+      <c r="A123" s="20" t="inlineStr">
         <is>
           <t>báo giá life english books</t>
         </is>
       </c>
-      <c r="B123" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C123" s="13" t="inlineStr"/>
-      <c r="D123" s="13" t="inlineStr">
+      <c r="B123" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C123" s="20" t="inlineStr"/>
+      <c r="D123" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E123" s="13" t="inlineStr"/>
-      <c r="F123" s="13" t="inlineStr"/>
+      <c r="E123" s="20" t="inlineStr"/>
+      <c r="F123" s="20" t="inlineStr"/>
+      <c r="G123" s="21" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="13" t="inlineStr">
+      <c r="A124" s="20" t="inlineStr">
         <is>
           <t>báo giá surface pro book</t>
         </is>
       </c>
-      <c r="B124" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C124" s="13" t="inlineStr"/>
-      <c r="D124" s="13" t="inlineStr">
+      <c r="B124" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C124" s="20" t="inlineStr"/>
+      <c r="D124" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E124" s="13" t="inlineStr"/>
-      <c r="F124" s="13" t="inlineStr"/>
+      <c r="E124" s="20" t="inlineStr"/>
+      <c r="F124" s="20" t="inlineStr"/>
+      <c r="G124" s="21" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="13" t="inlineStr">
+      <c r="A125" s="20" t="inlineStr">
         <is>
           <t>chặn thông báo face book đến mail</t>
         </is>
       </c>
-      <c r="B125" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C125" s="13" t="inlineStr"/>
-      <c r="D125" s="13" t="inlineStr">
+      <c r="B125" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C125" s="20" t="inlineStr"/>
+      <c r="D125" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E125" s="13" t="inlineStr"/>
-      <c r="F125" s="13" t="inlineStr"/>
+      <c r="E125" s="20" t="inlineStr"/>
+      <c r="F125" s="20" t="inlineStr"/>
+      <c r="G125" s="21" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" s="13" t="inlineStr">
+      <c r="A126" s="20" t="inlineStr">
         <is>
           <t>cài đặt tắt chuông báo face book</t>
         </is>
       </c>
-      <c r="B126" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C126" s="13" t="inlineStr"/>
-      <c r="D126" s="13" t="inlineStr">
+      <c r="B126" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C126" s="20" t="inlineStr"/>
+      <c r="D126" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E126" s="13" t="inlineStr"/>
-      <c r="F126" s="13" t="inlineStr"/>
+      <c r="E126" s="20" t="inlineStr"/>
+      <c r="F126" s="20" t="inlineStr"/>
+      <c r="G126" s="21" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" s="13" t="inlineStr">
+      <c r="A127" s="20" t="inlineStr">
         <is>
           <t>các câu thông báo bán hàng trên face book</t>
         </is>
       </c>
-      <c r="B127" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C127" s="13" t="inlineStr"/>
-      <c r="D127" s="13" t="inlineStr">
+      <c r="B127" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C127" s="20" t="inlineStr"/>
+      <c r="D127" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E127" s="13" t="inlineStr"/>
-      <c r="F127" s="13" t="inlineStr"/>
+      <c r="E127" s="20" t="inlineStr"/>
+      <c r="F127" s="20" t="inlineStr"/>
+      <c r="G127" s="21" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" s="13" t="inlineStr">
+      <c r="A128" s="20" t="inlineStr">
         <is>
           <t>cách tắt thông báo sinh nhật cho face book</t>
         </is>
       </c>
-      <c r="B128" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C128" s="13" t="inlineStr"/>
-      <c r="D128" s="13" t="inlineStr">
+      <c r="B128" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C128" s="20" t="inlineStr"/>
+      <c r="D128" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E128" s="13" t="inlineStr"/>
-      <c r="F128" s="13" t="inlineStr"/>
+      <c r="E128" s="20" t="inlineStr"/>
+      <c r="F128" s="20" t="inlineStr"/>
+      <c r="G128" s="21" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" s="13" t="inlineStr">
+      <c r="A129" s="20" t="inlineStr">
         <is>
           <t>email thông báo cho khách số booking khách sạn</t>
         </is>
       </c>
-      <c r="B129" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C129" s="13" t="inlineStr"/>
-      <c r="D129" s="13" t="inlineStr">
+      <c r="B129" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C129" s="20" t="inlineStr"/>
+      <c r="D129" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E129" s="13" t="inlineStr"/>
-      <c r="F129" s="13" t="inlineStr"/>
+      <c r="E129" s="20" t="inlineStr"/>
+      <c r="F129" s="20" t="inlineStr"/>
+      <c r="G129" s="21" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" s="13" t="inlineStr">
+      <c r="A130" s="20" t="inlineStr">
         <is>
           <t>face book báo không thể thay đổi tên trang</t>
         </is>
       </c>
-      <c r="B130" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C130" s="13" t="inlineStr"/>
-      <c r="D130" s="13" t="inlineStr">
+      <c r="B130" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C130" s="20" t="inlineStr"/>
+      <c r="D130" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E130" s="13" t="inlineStr"/>
-      <c r="F130" s="13" t="inlineStr"/>
+      <c r="E130" s="20" t="inlineStr"/>
+      <c r="F130" s="20" t="inlineStr"/>
+      <c r="G130" s="21" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" s="13" t="inlineStr">
+      <c r="A131" s="20" t="inlineStr">
         <is>
           <t>face book báo lỗi vi phạm tiêu chuẩn cộng động</t>
         </is>
       </c>
-      <c r="B131" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C131" s="13" t="inlineStr"/>
-      <c r="D131" s="13" t="inlineStr">
+      <c r="B131" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C131" s="20" t="inlineStr"/>
+      <c r="D131" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E131" s="13" t="inlineStr"/>
-      <c r="F131" s="13" t="inlineStr"/>
+      <c r="E131" s="20" t="inlineStr"/>
+      <c r="F131" s="20" t="inlineStr"/>
+      <c r="G131" s="21" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" s="13" t="inlineStr">
+      <c r="A132" s="20" t="inlineStr">
         <is>
           <t>face book báo something went wrong là bị gì</t>
         </is>
       </c>
-      <c r="B132" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C132" s="13" t="inlineStr"/>
-      <c r="D132" s="13" t="inlineStr">
+      <c r="B132" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C132" s="20" t="inlineStr"/>
+      <c r="D132" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E132" s="13" t="inlineStr"/>
-      <c r="F132" s="13" t="inlineStr"/>
+      <c r="E132" s="20" t="inlineStr"/>
+      <c r="F132" s="20" t="inlineStr"/>
+      <c r="G132" s="21" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="13" t="inlineStr">
+      <c r="A133" s="20" t="inlineStr">
         <is>
           <t>face book báo đổi mật khẩu</t>
         </is>
       </c>
-      <c r="B133" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C133" s="13" t="inlineStr"/>
-      <c r="D133" s="13" t="inlineStr">
+      <c r="B133" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C133" s="20" t="inlineStr"/>
+      <c r="D133" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E133" s="13" t="inlineStr"/>
-      <c r="F133" s="13" t="inlineStr"/>
+      <c r="E133" s="20" t="inlineStr"/>
+      <c r="F133" s="20" t="inlineStr"/>
+      <c r="G133" s="21" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" s="13" t="inlineStr">
+      <c r="A134" s="20" t="inlineStr">
         <is>
           <t>face book bị báo cáo mạo danh</t>
         </is>
       </c>
-      <c r="B134" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C134" s="13" t="inlineStr"/>
-      <c r="D134" s="13" t="inlineStr">
+      <c r="B134" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C134" s="20" t="inlineStr"/>
+      <c r="D134" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E134" s="13" t="inlineStr"/>
-      <c r="F134" s="13" t="inlineStr"/>
+      <c r="E134" s="20" t="inlineStr"/>
+      <c r="F134" s="20" t="inlineStr"/>
+      <c r="G134" s="21" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="13" t="inlineStr">
+      <c r="A135" s="20" t="inlineStr">
         <is>
           <t>face book của nhà báo hoàng nguyên vũ</t>
         </is>
       </c>
-      <c r="B135" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C135" s="13" t="inlineStr"/>
-      <c r="D135" s="13" t="inlineStr">
+      <c r="B135" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C135" s="20" t="inlineStr"/>
+      <c r="D135" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E135" s="13" t="inlineStr"/>
-      <c r="F135" s="13" t="inlineStr"/>
+      <c r="E135" s="20" t="inlineStr"/>
+      <c r="F135" s="20" t="inlineStr"/>
+      <c r="G135" s="21" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" s="13" t="inlineStr">
+      <c r="A136" s="20" t="inlineStr">
         <is>
           <t>hiển thị thông báo của face book chrome</t>
         </is>
       </c>
-      <c r="B136" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C136" s="13" t="inlineStr"/>
-      <c r="D136" s="13" t="inlineStr">
+      <c r="B136" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C136" s="20" t="inlineStr"/>
+      <c r="D136" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E136" s="13" t="inlineStr"/>
-      <c r="F136" s="13" t="inlineStr"/>
+      <c r="E136" s="20" t="inlineStr"/>
+      <c r="F136" s="20" t="inlineStr"/>
+      <c r="G136" s="21" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" s="13" t="inlineStr">
+      <c r="A137" s="20" t="inlineStr">
         <is>
           <t>huong dân xóa thông báo trên face book</t>
         </is>
       </c>
-      <c r="B137" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C137" s="13" t="inlineStr"/>
-      <c r="D137" s="13" t="inlineStr">
+      <c r="B137" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C137" s="20" t="inlineStr"/>
+      <c r="D137" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E137" s="13" t="inlineStr"/>
-      <c r="F137" s="13" t="inlineStr"/>
+      <c r="E137" s="20" t="inlineStr"/>
+      <c r="F137" s="20" t="inlineStr"/>
+      <c r="G137" s="21" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="13" t="inlineStr">
+      <c r="A138" s="20" t="inlineStr">
         <is>
           <t>hướng dẫn xóa thông báo trên face book</t>
         </is>
       </c>
-      <c r="B138" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C138" s="13" t="inlineStr"/>
-      <c r="D138" s="13" t="inlineStr">
+      <c r="B138" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C138" s="20" t="inlineStr"/>
+      <c r="D138" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E138" s="13" t="inlineStr"/>
-      <c r="F138" s="13" t="inlineStr"/>
+      <c r="E138" s="20" t="inlineStr"/>
+      <c r="F138" s="20" t="inlineStr"/>
+      <c r="G138" s="21" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" s="13" t="inlineStr">
+      <c r="A139" s="20" t="inlineStr">
         <is>
           <t>không nhận thông báo mời chơi game từ face book</t>
         </is>
       </c>
-      <c r="B139" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C139" s="13" t="inlineStr"/>
-      <c r="D139" s="13" t="inlineStr">
+      <c r="B139" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C139" s="20" t="inlineStr"/>
+      <c r="D139" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E139" s="13" t="inlineStr"/>
-      <c r="F139" s="13" t="inlineStr"/>
+      <c r="E139" s="20" t="inlineStr"/>
+      <c r="F139" s="20" t="inlineStr"/>
+      <c r="G139" s="21" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="13" t="inlineStr">
+      <c r="A140" s="20" t="inlineStr">
         <is>
           <t>không vào được face book báo lỗi proxy</t>
         </is>
       </c>
-      <c r="B140" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C140" s="13" t="inlineStr"/>
-      <c r="D140" s="13" t="inlineStr">
+      <c r="B140" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C140" s="20" t="inlineStr"/>
+      <c r="D140" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E140" s="13" t="inlineStr"/>
-      <c r="F140" s="13" t="inlineStr"/>
+      <c r="E140" s="20" t="inlineStr"/>
+      <c r="F140" s="20" t="inlineStr"/>
+      <c r="G140" s="21" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" s="13" t="inlineStr">
+      <c r="A141" s="20" t="inlineStr">
         <is>
           <t>laàm sao biết ai báo cáo tên face book</t>
         </is>
       </c>
-      <c r="B141" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C141" s="13" t="inlineStr"/>
-      <c r="D141" s="13" t="inlineStr">
+      <c r="B141" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C141" s="20" t="inlineStr"/>
+      <c r="D141" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E141" s="13" t="inlineStr"/>
-      <c r="F141" s="13" t="inlineStr"/>
+      <c r="E141" s="20" t="inlineStr"/>
+      <c r="F141" s="20" t="inlineStr"/>
+      <c r="G141" s="21" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="13" t="inlineStr">
+      <c r="A142" s="20" t="inlineStr">
         <is>
           <t>my book live báo đèn đỏ</t>
         </is>
       </c>
-      <c r="B142" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C142" s="13" t="inlineStr"/>
-      <c r="D142" s="13" t="inlineStr">
+      <c r="B142" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C142" s="20" t="inlineStr"/>
+      <c r="D142" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E142" s="13" t="inlineStr"/>
-      <c r="F142" s="13" t="inlineStr"/>
+      <c r="E142" s="20" t="inlineStr"/>
+      <c r="F142" s="20" t="inlineStr"/>
+      <c r="G142" s="21" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" s="13" t="inlineStr">
+      <c r="A143" s="20" t="inlineStr">
         <is>
           <t>nghiệp vụ báo giá và xác nhận booking note</t>
         </is>
       </c>
-      <c r="B143" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C143" s="13" t="inlineStr"/>
-      <c r="D143" s="13" t="inlineStr">
+      <c r="B143" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C143" s="20" t="inlineStr"/>
+      <c r="D143" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E143" s="13" t="inlineStr"/>
-      <c r="F143" s="13" t="inlineStr"/>
+      <c r="E143" s="20" t="inlineStr"/>
+      <c r="F143" s="20" t="inlineStr"/>
+      <c r="G143" s="21" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="13" t="inlineStr">
+      <c r="A144" s="20" t="inlineStr">
         <is>
           <t>statement of books báo cáo sổ sách</t>
         </is>
       </c>
-      <c r="B144" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C144" s="13" t="inlineStr"/>
-      <c r="D144" s="13" t="inlineStr">
+      <c r="B144" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C144" s="20" t="inlineStr"/>
+      <c r="D144" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E144" s="13" t="inlineStr"/>
-      <c r="F144" s="13" t="inlineStr"/>
+      <c r="E144" s="20" t="inlineStr"/>
+      <c r="F144" s="20" t="inlineStr"/>
+      <c r="G144" s="21" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="13" t="inlineStr">
+      <c r="A145" s="20" t="inlineStr">
         <is>
           <t>style book của tờ báo</t>
         </is>
       </c>
-      <c r="B145" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C145" s="13" t="inlineStr"/>
-      <c r="D145" s="13" t="inlineStr">
+      <c r="B145" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C145" s="20" t="inlineStr"/>
+      <c r="D145" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E145" s="13" t="inlineStr"/>
-      <c r="F145" s="13" t="inlineStr"/>
+      <c r="E145" s="20" t="inlineStr"/>
+      <c r="F145" s="20" t="inlineStr"/>
+      <c r="G145" s="21" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" s="13" t="inlineStr">
+      <c r="A146" s="20" t="inlineStr">
         <is>
           <t>thoông báo khai trương face book the coffee house</t>
         </is>
       </c>
-      <c r="B146" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C146" s="13" t="inlineStr"/>
-      <c r="D146" s="13" t="inlineStr">
+      <c r="B146" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C146" s="20" t="inlineStr"/>
+      <c r="D146" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E146" s="13" t="inlineStr"/>
-      <c r="F146" s="13" t="inlineStr"/>
+      <c r="E146" s="20" t="inlineStr"/>
+      <c r="F146" s="20" t="inlineStr"/>
+      <c r="G146" s="21" t="inlineStr"/>
     </row>
     <row r="147">
-      <c r="A147" s="13" t="inlineStr">
+      <c r="A147" s="20" t="inlineStr">
         <is>
           <t>thông báo khi booking trong wordpress</t>
         </is>
       </c>
-      <c r="B147" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C147" s="13" t="inlineStr"/>
-      <c r="D147" s="13" t="inlineStr">
+      <c r="B147" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C147" s="20" t="inlineStr"/>
+      <c r="D147" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E147" s="13" t="inlineStr"/>
-      <c r="F147" s="13" t="inlineStr"/>
+      <c r="E147" s="20" t="inlineStr"/>
+      <c r="F147" s="20" t="inlineStr"/>
+      <c r="G147" s="21" t="inlineStr"/>
     </row>
     <row r="148">
-      <c r="A148" s="13" t="inlineStr">
+      <c r="A148" s="20" t="inlineStr">
         <is>
           <t>thông báo messenger khi book trong wordpress</t>
         </is>
       </c>
-      <c r="B148" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C148" s="13" t="inlineStr"/>
-      <c r="D148" s="13" t="inlineStr">
+      <c r="B148" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C148" s="20" t="inlineStr"/>
+      <c r="D148" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E148" s="13" t="inlineStr"/>
-      <c r="F148" s="13" t="inlineStr"/>
+      <c r="E148" s="20" t="inlineStr"/>
+      <c r="F148" s="20" t="inlineStr"/>
+      <c r="G148" s="21" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" s="13" t="inlineStr">
+      <c r="A149" s="20" t="inlineStr">
         <is>
           <t>thông báo thông báo khi book trong wordpress</t>
         </is>
       </c>
-      <c r="B149" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C149" s="13" t="inlineStr"/>
-      <c r="D149" s="13" t="inlineStr">
+      <c r="B149" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C149" s="20" t="inlineStr"/>
+      <c r="D149" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E149" s="13" t="inlineStr"/>
-      <c r="F149" s="13" t="inlineStr"/>
+      <c r="E149" s="20" t="inlineStr"/>
+      <c r="F149" s="20" t="inlineStr"/>
+      <c r="G149" s="21" t="inlineStr"/>
     </row>
     <row r="150">
-      <c r="A150" s="13" t="inlineStr">
+      <c r="A150" s="20" t="inlineStr">
         <is>
           <t>thông báo về việc giao nhận booking trễ</t>
         </is>
       </c>
-      <c r="B150" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C150" s="13" t="inlineStr"/>
-      <c r="D150" s="13" t="inlineStr">
+      <c r="B150" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C150" s="20" t="inlineStr"/>
+      <c r="D150" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E150" s="13" t="inlineStr"/>
-      <c r="F150" s="13" t="inlineStr"/>
+      <c r="E150" s="20" t="inlineStr"/>
+      <c r="F150" s="20" t="inlineStr"/>
+      <c r="G150" s="21" t="inlineStr"/>
     </row>
     <row r="151">
-      <c r="A151" s="13" t="inlineStr">
+      <c r="A151" s="20" t="inlineStr">
         <is>
           <t>thông báo đien lực đức thọ fa book hà tinh</t>
         </is>
       </c>
-      <c r="B151" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C151" s="13" t="inlineStr"/>
-      <c r="D151" s="13" t="inlineStr">
+      <c r="B151" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C151" s="20" t="inlineStr"/>
+      <c r="D151" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E151" s="13" t="inlineStr"/>
-      <c r="F151" s="13" t="inlineStr"/>
+      <c r="E151" s="20" t="inlineStr"/>
+      <c r="F151" s="20" t="inlineStr"/>
+      <c r="G151" s="21" t="inlineStr"/>
     </row>
     <row r="152">
-      <c r="A152" s="13" t="inlineStr">
+      <c r="A152" s="20" t="inlineStr">
         <is>
           <t>thông cáo báo chí thái hà books</t>
         </is>
       </c>
-      <c r="B152" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C152" s="13" t="inlineStr"/>
-      <c r="D152" s="13" t="inlineStr">
+      <c r="B152" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C152" s="20" t="inlineStr"/>
+      <c r="D152" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E152" s="13" t="inlineStr"/>
-      <c r="F152" s="13" t="inlineStr"/>
+      <c r="E152" s="20" t="inlineStr"/>
+      <c r="F152" s="20" t="inlineStr"/>
+      <c r="G152" s="21" t="inlineStr"/>
     </row>
     <row r="153">
-      <c r="A153" s="13" t="inlineStr">
+      <c r="A153" s="20" t="inlineStr">
         <is>
           <t>tạo tin báo trong face book</t>
         </is>
       </c>
-      <c r="B153" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C153" s="13" t="inlineStr"/>
-      <c r="D153" s="13" t="inlineStr">
+      <c r="B153" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C153" s="20" t="inlineStr"/>
+      <c r="D153" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E153" s="13" t="inlineStr"/>
-      <c r="F153" s="13" t="inlineStr"/>
+      <c r="E153" s="20" t="inlineStr"/>
+      <c r="F153" s="20" t="inlineStr"/>
+      <c r="G153" s="21" t="inlineStr"/>
     </row>
     <row r="154">
-      <c r="A154" s="13" t="inlineStr">
+      <c r="A154" s="20" t="inlineStr">
         <is>
           <t>tắt thông báo bằng mail của booking và agoda</t>
         </is>
       </c>
-      <c r="B154" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C154" s="13" t="inlineStr"/>
-      <c r="D154" s="13" t="inlineStr">
+      <c r="B154" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C154" s="20" t="inlineStr"/>
+      <c r="D154" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E154" s="13" t="inlineStr"/>
-      <c r="F154" s="13" t="inlineStr"/>
+      <c r="E154" s="20" t="inlineStr"/>
+      <c r="F154" s="20" t="inlineStr"/>
+      <c r="G154" s="21" t="inlineStr"/>
     </row>
     <row r="155">
-      <c r="A155" s="13" t="inlineStr">
+      <c r="A155" s="20" t="inlineStr">
         <is>
           <t>tắt thông báo mini face book</t>
         </is>
       </c>
-      <c r="B155" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C155" s="13" t="inlineStr"/>
-      <c r="D155" s="13" t="inlineStr">
+      <c r="B155" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C155" s="20" t="inlineStr"/>
+      <c r="D155" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E155" s="13" t="inlineStr"/>
-      <c r="F155" s="13" t="inlineStr"/>
+      <c r="E155" s="20" t="inlineStr"/>
+      <c r="F155" s="20" t="inlineStr"/>
+      <c r="G155" s="21" t="inlineStr"/>
     </row>
     <row r="156">
-      <c r="A156" s="13" t="inlineStr">
+      <c r="A156" s="20" t="inlineStr">
         <is>
           <t>tắtht ông báo live strem và video trên face book</t>
         </is>
       </c>
-      <c r="B156" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C156" s="13" t="inlineStr"/>
-      <c r="D156" s="13" t="inlineStr">
+      <c r="B156" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C156" s="20" t="inlineStr"/>
+      <c r="D156" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E156" s="13" t="inlineStr"/>
-      <c r="F156" s="13" t="inlineStr"/>
+      <c r="E156" s="20" t="inlineStr"/>
+      <c r="F156" s="20" t="inlineStr"/>
+      <c r="G156" s="21" t="inlineStr"/>
     </row>
     <row r="157">
-      <c r="A157" s="13" t="inlineStr">
+      <c r="A157" s="20" t="inlineStr">
         <is>
           <t>vacpa e book báo cáo tài chính</t>
         </is>
       </c>
-      <c r="B157" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C157" s="13" t="inlineStr"/>
-      <c r="D157" s="13" t="inlineStr">
+      <c r="B157" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C157" s="20" t="inlineStr"/>
+      <c r="D157" s="20" t="inlineStr">
         <is>
           <t>Z. Rác - không liên quan</t>
         </is>
       </c>
-      <c r="E157" s="13" t="inlineStr"/>
-      <c r="F157" s="13" t="inlineStr"/>
+      <c r="E157" s="20" t="inlineStr"/>
+      <c r="F157" s="20" t="inlineStr"/>
+      <c r="G157" s="21" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F157"/>
+  <autoFilter ref="A1:G157"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>

</xml_diff>

<commit_message>
auto: session 2026-08-05 14:11
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
+++ b/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Backlink dofollow/nofollow (~50%); SEO/Entity/Guest Post/Textlink; số đầu báo hợp tác (200+/300+/1000+); DR/DA (hiếm - đa số đối thủ KHÔNG có số thật); tên báo core: VnExpress, Dân Trí, CafeF, 24h, Kênh14, VietNamNet, Tuổi Trẻ; phân loại báo lớn/tỉnh/ngành/đảng; giá theo bài, số từ 800-1200, số ảnh, thời gian đăng, chiết khấu; AEO/GEO (hiếm, 1/15 - cơ hội khác biệt)</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       <c r="F38" s="5" t="inlineStr"/>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       <c r="F43" s="5" t="inlineStr"/>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       <c r="F44" s="5" t="inlineStr"/>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Giá bài PR theo hạng/vị trí (10,5-60tr/bài, phổ biến 15-50tr); Backlink/dofollow/DR-DA (12/15); giới hạn ≤1000 từ, 1-3 ảnh, tiêu đề 13-14 từ, lead ≤32 từ; thời gian duyệt 24-48h; vị trí đăng (trang chủ/box nổi bật/chuyên mục con); traffic/pageview thật của báo; Entity/Guest Post/Native Ads; giới hạn số link/bài (tối đa 2)</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2518,7 @@
       <c r="F70" s="8" t="inlineStr"/>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       <c r="F71" s="8" t="inlineStr"/>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
       <c r="F72" s="8" t="inlineStr"/>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       <c r="F73" s="8" t="inlineStr"/>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       <c r="F74" s="8" t="inlineStr"/>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       <c r="F75" s="8" t="inlineStr"/>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       <c r="F76" s="8" t="inlineStr"/>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       <c r="F77" s="8" t="inlineStr"/>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
       <c r="F78" s="8" t="inlineStr"/>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
       <c r="F79" s="8" t="inlineStr"/>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2750,7 @@
       <c r="F80" s="8" t="inlineStr"/>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       <c r="F81" s="8" t="inlineStr"/>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       <c r="F82" s="8" t="inlineStr"/>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2819,7 @@
       <c r="F83" s="8" t="inlineStr"/>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>Booking Fanpage; Booking KOLs/KOCs/Influencer; Banner quảng cáo (chuẩn IAB 300x250/728x90/160x600); TVC 10-30s; Livestream; Media Booking/Media Plan; Textlink; tier KOL Nano/Micro/Mid/Macro/Mega/Celeb; CPM/CPC/CPV/CPL; Engagement Rate; Reach; Follower; giá VNĐ/post (LƯU Ý: dịch vụ này Digicom CHƯA bán)</t>
+          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       <c r="F84" s="10" t="inlineStr"/>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       <c r="F85" s="10" t="inlineStr"/>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       <c r="F86" s="10" t="inlineStr"/>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2911,7 @@
       <c r="F87" s="10" t="inlineStr"/>
       <c r="G87" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -2934,7 +2934,7 @@
       <c r="F88" s="10" t="inlineStr"/>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       <c r="F89" s="10" t="inlineStr"/>
       <c r="G89" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       <c r="F90" s="10" t="inlineStr"/>
       <c r="G90" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       <c r="F91" s="10" t="inlineStr"/>
       <c r="G91" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="F92" s="10" t="inlineStr"/>
       <c r="G92" s="11" t="inlineStr">
         <is>
-          <t>Quy trình 5-6 bước (tiếp brief → chọn đầu báo/chuyên mục → viết bài PR → duyệt &amp; ký HĐ → đăng → nghiệm thu); Backlink (5/15); DR/UR/Ahrefs; Advertorial; báo core VnExpress/Dân Trí/VietNamNet/Kênh14/24h; chuẩn bài 1000 từ + 5 ảnh, 1-3 link; giá 700k-150tr/bài theo tier báo; đăng 1-14 ngày; 200-1000+ đầu báo hợp tác; GAP: chưa đối thủ nào hướng dẫn DIY tự liên hệ toà soạn, chưa ai nhắc Điều 38 Luật Báo chí</t>
+          <t>NGHIÊN CỨU 8 nguồn (WebSearch 8 truy vấn + WebFetch 5 trang chi tiết). Quy trình 6 bước lặp lại nhiều nhất (3/5 nguồn nêu đủ 6 bước): (1) Tiếp nhận nhu cầu/chốt brief (mục tiêu, độc giả, timeline, ngân sách, loại nội dung PR/advertorial/phỏng vấn); (2) Tư vấn/chọn đầu báo &amp; chuyên mục phù hợp; (3) Lập hợp đồng, thoả thuận hình thức thanh toán (trước/sau đăng); (4) Chuẩn bị nội dung + gửi duyệt + chỉnh sửa theo phản hồi toà soạn (đổi tiêu đề, rút gọn, đổi ảnh, giảm 'màu quảng cáo'); (5) Book bài, chốt lịch/giờ đăng, giám sát tiến độ; (6) Nghiệm thu (đối chiếu tiêu đề/nội dung/hình ảnh/link với bản duyệt, lưu chứng từ) + thanh toán phần còn lại/báo cáo. Hợp đồng: lập hợp đồng dịch vụ, gửi bản mềm cho khách duyệt trước khi ký (2/5 nguồn). Hoá đơn VAT: xuất SAU khi khách thanh toán đủ, nếu khách yêu cầu (1/5 nguồn) - lưu ý quy định thuế chung liên quan (không đặc thù ngành báo): hoá đơn từ 5 triệu đồng trở lên phải thanh toán chuyển khoản mới được khấu trừ thuế, GAP - hầu như không agency nào trong ngành nhắc quy định này dù rất liên quan khách B2B. Backlink/DR/UR/Ahrefs (nhóm riêng, chỉ xuất hiện ở site chuyên SEO offpage như DanaSEO, không trộn với bài how-to booking thuần PR): quy trình đặt backlink báo PR gồm chọn báo uy tín -&gt; viết nội dung chuẩn SEO + anchor text tự nhiên -&gt; submit URL Google Search Console để index nhanh -&gt; theo dõi bằng Ahrefs/GSC/SEMrush; DR đánh giá độ tin cậy toàn domain, UR đánh giá riêng URL chứa backlink; DR/UR thường tăng ngay 3-7 ngày sau đăng. GAP: các bài how-to booking báo thuần PR hầu như KHÔNG nhắc DR/UR/Ahrefs - cơ hội gộp 2 góc 'PR thương hiệu' + 'SEO backlink' trong 1 bài mà đối thủ booking thuần chưa làm. Loại hình báo: các nguồn phân loại theo mục tiêu chứ không theo giấy/điện tử/tạp chí rõ ràng ('báo điện tử tổng hợp' = độ phủ nhanh, 'báo chính thống' = uy tín thương hiệu, 'báo chuyên ngành' = đúng tệp target) - GAP: không nguồn nào phân tách rõ 3 loại hình báo giấy/tạp chí/điện tử với đặc thù riêng (báo giấy cần duyệt bản in, tạp chí có chu kỳ phát hành khác điện tử). Chuẩn bài PR: chỉ 1/5 nguồn nêu con số cụ thể '1.000 từ + 5 ảnh là chuẩn phổ biến, 1-2 hyperlink tuỳ báo, video tính phí thêm từ 2 triệu' - các nguồn khác chỉ nói chung chung 'chuẩn theo quy định từng báo' - GAP lớn, Digicom hiện đã có bảng giá + field 'yêu cầu' cụ thể theo từng đầu báo (số ảnh, số link, độ dài) là điểm khác biệt info gain thật. Nội dung bài PR chuẩn: mở bài cuốn hút -&gt; thân bài rõ ràng -&gt; có quote/trích dẫn đại diện DN -&gt; có số liệu -&gt; kết bài CTA nhẹ, kèm ảnh/logo/infographic chất lượng cao; tiêu đề phải trung tính, tránh giọng quảng cáo hô hào, tránh viết như tờ rơi (lưu ý được lặp lại nhiều nhất). Thời gian triển khai: tối thiểu 1 ngày làm việc để đăng bài (1 nguồn, không nguồn nào khác nêu con số). Ngành hàng phù hợp (chỉ 1 nguồn nêu): F&amp;B/nhà hàng, Beauty &amp; Spa, Giáo dục, Bất động sản, Máy móc công nghiệp - GAP: hầu hết bài how-to KHÔNG map rõ loại chiến lược PR nào hợp ngành nào - cơ hội làm bảng mapping ngành x loại báo/tier. SEO/backlink, GEO/AEO: chỉ 1 nguồn nhắc nhẹ audit intent/silo/internal link (không hẳn về booking báo) - HOÀN TOÀN KHÔNG có nguồn nào (0/8) nhắc GEO/AEO dù là xu hướng 2026. PR/thương hiệu, khủng hoảng truyền thông: các nguồn chỉ nói chung 'tăng độ phủ, tăng uy tín, ra mắt sản phẩm' - KHÔNG nguồn nào bàn về khủng hoảng truyền thông/xử lý khủng hoảng qua booking báo - GAP, có thể là góc content riêng (PR phòng ngừa khủng hoảng, đính chính thông tin). Hành vi khách hàng - DIY, pháp lý: không nguồn nào bàn việc DN tự liên hệ toà soạn (DIY) thay vì qua agency - GAP. CẢNH BÁO PHÁP LÝ QUAN TRỌNG (cần xử lý ngay trên site): điều luật đúng về 'Quảng cáo trên báo chí' là ĐIỀU 44 Luật Báo chí 2016, KHÔNG PHẢI Điều 38 (Điều 38 thực chất là 'Cung cấp thông tin cho báo chí', khác chủ đề hoàn toàn). Nội dung cũ/kế hoạch cũ của digicomvn.com từng định hướng nhắc 'Điều 38 Luật Báo chí' cho ngữ cảnh quảng cáo - CẦN RÀ LẠI VÀ SỬA THÀNH ĐIỀU 44 nếu đã hoặc sắp xuất bản, đối chiếu luatvietnam.vn trước khi dùng (theo rule content-professional.md - không claim sai luật). NGUỒN: medialabs.asia, quangbathuonghieu.vn, guestpost.com.vn, itify.vn, danaseo.net (2 bài), marketingai.vn, tcteamcorp.com, sapo.vn (quy định VAT chung), luatvietnam.vn (xác minh điều luật).</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3049,7 @@
       <c r="F93" s="12" t="inlineStr"/>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
       <c r="F94" s="12" t="inlineStr"/>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       <c r="F95" s="12" t="inlineStr"/>
       <c r="G95" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       <c r="F96" s="12" t="inlineStr"/>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       <c r="F97" s="12" t="inlineStr"/>
       <c r="G97" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
       <c r="F98" s="12" t="inlineStr"/>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       <c r="F99" s="12" t="inlineStr"/>
       <c r="G99" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       <c r="F100" s="12" t="inlineStr"/>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       <c r="F101" s="12" t="inlineStr"/>
       <c r="G101" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
       <c r="F102" s="12" t="inlineStr"/>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>Chiết khấu đại lý/agency 10-50%; white-label backlink báo; đầu báo core VnExpress/Dân Trí/Kênh14/24h/CafeF/Tuổi Trẻ/Thanh Niên/VietNamNet; Backlink/dofollow-nofollow/UR-DR (Ahrefs); tier báo (Loại 1-6, VIP); Advertorial; SLA; Guest Post; giá/bài 200k-15tr; 800-1200 từ; ngân sách tối thiểu (vd 50tr/tháng); báo Đảng/chuyên ngành; GAP: chưa ai công khai MOQ (số lượng tối thiểu) để hưởng chiết khấu</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="G104" s="16" t="inlineStr">
         <is>
-          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="G106" s="16" t="inlineStr">
         <is>
-          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>Booking PR/bài PR báo điện tử; Guest Post; Backlink báo (dofollow/nofollow); Social Entity/Entity Building; Textlink; Banner; TVC; UR/DR; Traffic/Pageviews; AEO/GEO (1/15, hiếm); đầu báo core VnExpress/Dân Trí/24h/VietNamNet/Kênh14/CafeF/Tuổi Trẻ/Thanh Niên; giá 500K-80tr/bài; 100-300+ đầu báo; 700-1200 từ; 2-5 ảnh; 1-3 link; hạng báo A/B/Top3/Đảng/tỉnh; vị trí trang chủ/chuyên mục; chiết khấu 10-35%</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G108" s="19" t="inlineStr">
         <is>
-          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="G109" s="19" t="inlineStr">
         <is>
-          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="G110" s="19" t="inlineStr">
         <is>
-          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="G111" s="19" t="inlineStr">
         <is>
-          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="G112" s="19" t="inlineStr">
         <is>
-          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="G113" s="19" t="inlineStr">
         <is>
-          <t>Booking báo PR quốc tế; Dofollow/Nofollow backlink; Guest post; PBN (Private Blog Network); DA; Permanent placement; tên báo đối thủ hay dùng: Digital Journal, ABC News, NBC News, Fox TV Stations (đài Mỹ hạng thấp - KHÔNG đối thủ nào thật sự có Forbes/CNN/Time/Business Insider/Yahoo Finance/MarketWatch - đây là GAP lớn nhất, Digicom có cơ hội khác biệt nếu xác minh được hợp tác thật); giá ~220-920 USD/gói; đăng 48h-10 ngày; bài tiếng Anh 600-800 từ; 1-5 text link/đầu báo; tier báo lớn/tỉnh/wire quốc tế</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: session 2026-08-05 14:13
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
+++ b/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn.</t>
+          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       <c r="F38" s="5" t="inlineStr"/>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       <c r="F43" s="5" t="inlineStr"/>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       <c r="F44" s="5" t="inlineStr"/>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com.</t>
+          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3049,7 @@
       <c r="F93" s="12" t="inlineStr"/>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
       <c r="F94" s="12" t="inlineStr"/>
       <c r="G94" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       <c r="F95" s="12" t="inlineStr"/>
       <c r="G95" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       <c r="F96" s="12" t="inlineStr"/>
       <c r="G96" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       <c r="F97" s="12" t="inlineStr"/>
       <c r="G97" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3164,7 @@
       <c r="F98" s="12" t="inlineStr"/>
       <c r="G98" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       <c r="F99" s="12" t="inlineStr"/>
       <c r="G99" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3210,7 @@
       <c r="F100" s="12" t="inlineStr"/>
       <c r="G100" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       <c r="F101" s="12" t="inlineStr"/>
       <c r="G101" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
       <c r="F102" s="12" t="inlineStr"/>
       <c r="G102" s="13" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet).</t>
+          <t>NGHIÊN CỨU 11 trang fetch được + 5 trang chỉ đọc qua snippet. Chiết khấu đại lý/agency: TCC &amp; Partners 20-40%; Life Media tới 40%; MIC Creative tới 50%; BookBáoPR 10-35% so với giá công bố; đa số agency (KMEDIA, SEODO, MIC Creative, Á Châu Media, Brandcom, Mona Media, Admicro) KHÔNG công khai % chiết khấu trên website, chỉ tư vấn riêng qua hotline/chat - GAP: content gap Digicom có thể khai thác (minh bạch % chiết khấu ngay trên trang). White-label: KHÔNG agency nào công khai nói 'white-label'/'gắn thương hiệu đại lý' - GAP rõ rệt dù đối tượng khách rõ ràng gồm cả agency trung gian mua lại để bán tiếp. MOQ (số lượng tối thiểu): không trang nào công bố số bài/tháng tối thiểu để hưởng giá đại lý - chỉ có 'ngân sách tối thiểu' dạng tiền (SEODO ~500k-1tr) - GAP, chưa ai công bố bảng MOQ theo số bài/tháng gắn % chiết khấu bậc thang. Tên đầu báo core (theo tần suất): VnExpress (nhiều nhất), Kênh14, Dân Trí, 24h.com.vn, Zing/Znews, Báo Mới, Soha, Thanh Niên, Tuổi Trẻ, VTC, CafeF, Batdongsan.com.vn, GameK. HapoDigital phân 2 hạng: Hạng A (soha.vn, baomoi.com, Zing.vn, Vnexpress, 24h, kenh14, Dantri) và Hạng B (thanhnien.vn, tuoitre.vn, batdongsan.com.vn, gamek + 20 báo khác không nêu tên). Giá cụ thể: 24h.com.vn từ 3,4tr, VnExpress từ 13,2tr, Kênh14 từ 7,2tr. Loại link dofollow/nofollow, UR/DR: nhấn mạnh 'backlink từ trang uy tín UR/DR cao' nhưng KHÔNG công bố số cụ thể theo từng báo - GAP lớn, Digicom hiện đã có sẵn dữ liệu DR thật (Ahrefs) theo bang-gia-booking.md - lợi thế cạnh tranh rõ so với thị trường. Tier báo: thị trường phổ biến dùng 'Hạng A/Hạng B' hoặc phân nhóm chức năng 'báo PR lớn/trung ương-Đảng' (VnExpress, VTC, Dân Trí), 'báo tỉnh - trực thuộc tỉnh ủy', 'báo tầm trung có dofollow' - chưa thấy agency nào công khai hệ tier số (1-6)/VIP - có thể là phân loại nội bộ chưa công bố. Advertorial: không trang nào dùng thuật ngữ tường minh, thị trường VN gọi chung 'bài PR'/'bài quảng bá sản phẩm, thương hiệu'. SLA: 1/5 nguồn (medialabs) nêu SLA là 1 trong 5 tiêu chí đánh giá agency ('tốc độ phản hồi và xử lý phát sinh'), tiêu chí thứ 5 là 'nghiệm thu' (proof rõ ràng: link, hình ảnh, thời gian) - 2 tiêu chí cốt lõi được nêu tường minh nhất. Hợp đồng, hoá đơn VAT: quy trình 5 bước có bước 'ký hợp đồng' (SEOViP, SEODO) nhưng KHÔNG nguồn nào nhắc cụ thể hoá đơn VAT/thuế công khai - GAP, điểm B2B thật sự cần nhưng thị trường không nói rõ ai xuất hoá đơn VAT. Giá/bài: dải rất rộng - SEOViP báo lớn 2tr/bài, báo tỉnh 1tr/bài, gói tiết kiệm 700k/bài, guest post thường 200k/bài; BookBáoPR 24h từ 3,4tr, Kênh14 từ 7,2tr, VnExpress từ 13,2tr; không agency nào nêu ngân sách tối thiểu THEO THÁNG cho khách agency/đại lý (chỉ theo đơn lẻ). Loại báo: 3 nhóm lặp lại nhất: báo lớn/trung ương gắn mác 'Đảng' (VnExpress, VTC, Dân Trí), báo tỉnh, báo tầm trung/chuyên ngành có dofollow; Admicro là agency duy nhất công khai có cả kênh báo giấy; không nguồn nào tách riêng 'tạp chí' như 1 nhóm riêng biệt. Ngành hàng phù hợp B2B agency: không nguồn nào liệt kê cụ thể ngoài gợi ý chung theo target audience (khách trẻ -&gt; báo online, khách trung niên/cao tuổi -&gt; báo giấy/tạp chí) - GAP về phân khúc ngành. PR/marketing/thương hiệu: 3 lợi ích chính lặp lại - tăng nhận diện thương hiệu, tăng uy tín/độ tin cậy, hỗ trợ traffic/doanh số; SEODO thêm use-case riêng: 'tích xanh xác thực trên mạng xã hội' nhờ bài báo uy tín làm bằng chứng. SEO/backlink/GEO/AEO: SEOViP nhấn SEO rõ nhất (UR/DR cao, traffic organic, thứ hạng Google); HapoDigital + BookBáoPR bán kèm backlink/entity building/guest post cùng gói booking - KHÔNG agency nào nhắc GEO/AEO - GAP hoàn toàn dù là xu hướng 2026. Hành vi B2B chọn nhà cung cấp (khung 5 tiêu chí rõ nhất, từ medialabs): (1) network báo chí - ưu tiên chất lượng hơn số lượng, (2) chi phí - xem toàn bộ cấu trúc giá chứ không chỉ giá niêm yết, (3) SLA - tốc độ phản hồi/xử lý phát sinh, (4) nội dung - năng lực biên tập + tuân thủ pháp lý, (5) nghiệm thu - proof rõ ràng; insight quan trọng: khách B2B KHÔNG chỉ chọn theo chiết khấu cao nhất mà cân bằng với SLA/chất lượng - Digicom nên định vị minh bạch SLA/proof nghiệm thu thay vì chỉ đua chiết khấu. Agency/đối thủ được nhắc tên (ghi nhận nội bộ, KHÔNG dùng để so sánh giá công khai trên trang bán hàng theo khong-ban-gov-edu.md/khong-link-doi-thu.md): MIC Creative, Admicro, Life Media, Brandcom, Mona Media, Á Châu Media, TCC &amp; Partners, SEODO, SEOViP, BookBáoPR, KMEDIA, HapoDigital, Ori Agency, Vion, TACO Media, ButVangCorp, DPS.Media. NGUỒN: accesstrade.vn, oriagency.vn, butvangcorp.com, medialabs.asia, seovip.vn, bookbaopr.vn, kmedia.vn, seodo.vn, miccreative.vn, hapodigital.com (tcc-agency.com lỗi DNS, 4 trang khác chỉ đọc qua snippet). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="G103" s="16" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="G104" s="16" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G105" s="16" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="G106" s="16" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="G107" s="16" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO).</t>
+          <t>NGHIÊN CỨU 10 trang (search 3 cụm từ khoá liên quan). Loại dịch vụ: Booking PR/đăng bài PR báo điện tử (10/10); Guest Post VN + quốc tế/Global (9/10); Backlink/link building/PBN system; Textlink; Banner quảng cáo; TVC/Video booking (3-6tr/clip 180s theo đầu báo); Social Entity; Toplist &amp; Review (bài xếp hạng Google); Content SEO writing/viết bài PR (300k-10tr/bài tuỳ cấp writer, bán riêng hoặc kèm gói); Audit kỹ thuật (technical audits); CRM quản lý chiến dịch linkbuilding. UR/DR/Traffic: nhắc theo mốc lượt truy cập cụ thể (gói cơ bản &lt;2.000 lượt/tháng, gói nâng cao &gt;10 triệu, gói toàn diện &gt;30 triệu); DR 20-80 cho site guest post (không phải báo điện tử); không agency nào công khai bảng UR/DR đầy đủ cho từng đầu báo lớn - chỉ nhắc ở mức market chung. AEO/GEO/LLMO: KHÔNG agency booking báo nào (0/10) nhắc trong trang bảng giá - khái niệm này chỉ xuất hiện ở blog SEO agency riêng biệt (Ori Marketing, Seodao, Sieutocviet, Tanphatdigital), hoàn toàn tách biệt khỏi thị trường booking báo/PR - góc Digicom CÓ THỂ khai thác làm điểm khác biệt. Đầu báo core (tần suất/10 nguồn): VnExpress (10, giá 10,5-230tr tuỳ vị trí, Top Story tới 150-230tr); Dân Trí (8); Kênh14 (7, từ 7,2tr); 24h.com.vn (7, từ 3,4tr đến 85tr); Tuổi Trẻ (6); Thanh Niên (5); Zing/ZNews (5); VietNamNet (4); Afamily.vn (3); CafeF/VnEconomy (3, 5-85tr); Tiền Phong (6-13tr); Hà Nội Mới (3-3,5tr); Đắk Lắk/Quảng Nam/Đà Nẵng - báo tỉnh (1,2-5,5tr); Đầu Tư Việt Nam (14-16tr); Advertising Vietnam - tạp chí ngành marketing (18-21tr). Giá/quy cách: dao động 700.000đ - 230 triệu đồng/bài tuỳ hạng báo và vị trí; quy cách phổ biến nhất '1.000 từ + 3-5 ảnh + 1-2 link'; số đầu báo hợp tác tự công bố: 200+ đến 1000+ báo (số liệu marketing, chưa kiểm chứng độc lập). Hạng báo/phân tầng: phổ biến 3 tầng - 'báo lớn/quốc gia' vs 'báo tỉnh/địa phương' vs 'báo dofollow tầm trung' (SEODO gọi thẳng 'Dofollow Newspapers'); có agency phân theo GÓI (Basic/Advanced/Comprehensive) gắn mốc traffic thay vì theo đầu báo; Guestpost.com.vn phân gói Basic/Premium/VIP/Agency theo số bài/tháng (9-150 bài, 2,5-40tr/tháng). Vị trí đăng: 'Trang chủ/Top Story' giá cao nhất; 'chuyên mục' giá trung bình; có nơi phân theo 'gói vị trí'. Chiết khấu: 10-35% so với giá công khai khi ký HĐ/mua số lượng lớn; có nơi chiết khấu leo thang 0%-&gt;20%-&gt;50% theo gói; có nơi 3% (từ 5tr) -&gt; 10% (từ 50tr+) leo thang theo tổng giá trị đơn. VAT/hoá đơn: chỉ 1 nguồn nói rõ 'giá cơ sở CHƯA bao gồm phí viết bài/up video/VAT' - các agency khác không đề cập rõ VAT trong nội dung crawl được. Loại hình báo: chủ yếu báo điện tử (100%); có nhắc 'Party Newspaper'/báo Đảng (đăng trên báo cơ quan nhà nước); KHÔNG nguồn nào tách riêng 'báo giấy'/'tạp chí in' - tạp chí ngành vẫn ở dạng online. Ngành hàng phù hợp: bất động sản, du lịch, công nghệ, y tế/sức khoẻ, làm đẹp, nội thất; danh sách ngành CẤM: rượu/thuốc lá, thực phẩm chức năng không phép, cờ bạc, nội dung vi phạm pháp luật/phỉ báng/quảng cáo sai sự thật. Nội dung/quy trình: quy trình 5 bước lặp lại (tiếp nhận yêu cầu -&gt; tư vấn báo giá -&gt; ký HĐ/thanh toán -&gt; đăng bài -&gt; báo cáo kết quả); thời gian xử lý 1-6 ngày tuỳ gói; tối thiểu gửi bài trước 2-3 ngày; nhấn mạnh bài đăng 'tồn tại vĩnh viễn' (permanent). Hành vi khách khi xem bảng giá: rõ ràng có hành vi SO SÁNH GIÁ giữa các agency (nhiều trang tự PR 'giá rẻ nhất', 'chiết khấu cao nhất' - cạnh tranh giá gay gắt); TÌM GÓI PHÙ HỢP NGÂN SÁCH rất rõ qua cấu trúc 3 tier thấp/vừa/cao; một số agency công khai cam kết hoàn tiền nếu không index ('100% index guarantee'). Chưa có ở bảng hiện tại của Digicom (gợi ý bổ sung nếu muốn hơn đối thủ): mốc 'cam kết index/hoàn tiền', phân tầng theo TRAFFIC cụ thể thay vì chỉ theo tên báo, góc AEO/GEO hoàn toàn chưa ai làm. NGUỒN: brando.vn (5 trang con theo đầu báo), chobao.vn, seovip.vn, seodo.vn, bookbaopr.vn, bookingpr.vn, miccreative.vn, famemedia.vn, thitruong.today, guestpost.com.vn, brandsvietnam.com (đối chiếu AEO/GEO). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G108" s="19" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="G109" s="19" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="G110" s="19" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="G111" s="19" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="G112" s="19" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="G113" s="19" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ).</t>
+          <t>NGHIÊN CỨU sâu 16 nguồn (4 agency VN hàng đầu về booking báo quốc tế + wire service quốc tế + bài phân tích 'as seen on'). Loại dịch vụ: Booking báo PR quốc tế; backlink/guest post quốc tế; PBN quốc tế (IAC Digital claim '300+ báo hạt giống' mang dấu hiệu PBN núp bóng PR); Press release distribution/wire service (KHÁC bản chất 'booking báo' kiểu VN - phân phối qua network tự động, không phải đặt bài trực tiếp toà soạn); Guaranteed placement vs Submission-only; DoFollow/Nofollow (đa số KHÔNG công khai rõ, gói cao cấp mới có dofollow trả phí riêng); Anchor text tuỳ chọn; Permanent placement (đa số claim vĩnh viễn nhưng không kiểm chứng được); DA/DR làm thước đo chính (không agency VN nào công bố DA cụ thể minh bạch, chỉ nói chung 'DR 30-80+'); 'As Seen On' trust badge - kỹ thuật marketing dùng logo CNN/Forbes/Fox dù bài thực chất đăng trên site vệ tinh/syndicate của mạng lưới đó, KHÔNG phải trang chính do toà soạn biên tập; Branded content/glorified press release; Earned media vs Paid media. TÊN BÁO/SITE QUỐC TẾ THẬT SỰ tìm được (qua wire service, KHÔNG qua agency VN): AP News (DA 91+, xuất hiện nhiều nhất); Yahoo Finance (DA 94+, qua network syndicate); MarketWatch (DA 94+, qua PRWeb/Newswire/King Newswire); Morning Star (DA 94+); Street Insider (DA 94+); Digital Journal (DA thấp-trung, giá rẻ 10-50 USD/bài, tần suất cao nhất trong nhóm 'báo hạng thấp'); Benzinga (DA 83, 15-90 USD/bài); AsiaOne (DA 83/DR 80, traffic 170K US, 2 backlink dofollow, ~60 USD/bài); Business Insider (chỉ qua network syndicate rẻ tiền 60-90 USD, KHÔNG phải bản chính businessinsider.com biên tập); NewsBreak, Newsmax, Google News, Bing News, Fox Business/CBS/CW7 (qua network TV syndicate), Nasdaq (qua Newswire.com 349-3.999 USD), Black Enterprise, Factiva, Vents Magazine (15 USD, chất lượng thấp); ITSReleased, PublicistPaper, BigNewsNetwork, BMTimes, ThePilotNews ('báo hạt giống' DA thấp mà 1 agency VN liệt kê - rõ ràng site vệ tinh/blog nhỏ, KHÔNG phải báo lớn thật). KIỂM TRA GAP CNN/Forbes/Time/Business Insider/Yahoo Finance/MarketWatch: đọc trực tiếp 4 agency VN hàng đầu (Mona Media, Brando, Ori Agency, IAC Digital) - KHÔNG agency nào claim/liệt kê cụ thể CNN hoặc Time; toàn bộ nội dung chỉ xoay quanh báo Việt Nam; 1 agency (IAC Digital) dùng tên gọi mơ hồ '300+ báo hạt giống quốc tế' nhưng ví dụ thực tế toàn site DA thấp/không tên tuổi - dấu hiệu rõ của PBN/spam núp bóng, KHÔNG phải báo lớn thật; 1 site khác (PR Global VN) tự nhận qua snippet Google 'đăng bài trên báo uy tín như Forbes' nhưng KHÔNG verify được nội dung đầy đủ do lỗi kết nối 2 lần - CẦN KIỂM TRA LẠI, không dùng làm căn cứ khi chưa xác minh. KẾT LUẬN GAP: Digicom có cơ hội THẬT nếu làm minh bạch: (1) phân biệt rõ 'báo chính CNN.com/Forbes.com biên tập tay' (không ai bán được, giá x chục nghìn USD, cực khó) với 'network syndicate gắn mác qua as-seen-on' (giá rẻ, dễ mua, KHÔNG phải bài biên tập thật - phải nói rõ với khách để tránh vi phạm content-professional.md); (2) không đối thủ VN nào công khai DA/DR minh bạch từng site - Digicom công khai DA thật là lợi thế; (3) TUYỆT ĐỐI KHÔNG bịa claim 'đã từng đăng CNN/Forbes thật' nếu chưa từng làm - nên định vị trung thực 'kết nối mạng lưới báo quốc tế uy tín (AP News, Yahoo Finance, MarketWatch, Digital Journal, Benzinga...)' thay vì nêu CNN/Forbes như cam kết. Giá USD/gói: Digital Journal 10-20 USD/bài (thấp nhất); Benzinga 15-90 USD/bài; AsiaOne ~60 USD/bài; combo Benzinga+Digital Journal+AP News 50-90 USD; King Newswire gói Yahoo (guaranteed) 400 USD/bài (450+ outlet, DA 91-94+); BrandPush 195-795 USD/bài + 40-80 USD phí viết; EIN Presswire 299-999 USD/bài; PRWeb 120-480 USD/bài; Newswire.com 349-3.999 USD/bài; PR Newswire (Cision) 195-249 USD phí thành viên/năm + 350-8.700 USD/release - tier cao nhất, uy tín nhất thị trường quốc tế; 24-7 Press Release 49-479 USD/bài. Bài tiếng Anh: chuẩn phổ biến nhất 500-1.000 từ/bài; số text link 1-5 tuỳ gói (thường 2-3, gói cao 5); 1 ảnh/video đại diện thường bắt buộc. Thời gian đăng: nhanh nhất same-day/24h; trung bình 24-72h; chậm nhất tới 365 ngày (cho phép giữ credit dùng dần); qua agency VN trung gian ghi nhận 10-15 ngày do 'duyệt biên tập viên + duyệt site'. Tier báo: Tier 1 - wire service lớn/uy tín nhất (PR Newswire/Cision, GlobeNewswire, Newswire.com), giá cao nhất; Tier 2 - network syndicate DA cao xác nhận được (Yahoo Finance, MarketWatch, AP News, DA 91-94+), gói guaranteed 200-500 USD; Tier 3 - site DA trung bình phổ biến giá rẻ (Digital Journal, Benzinga, AsiaOne, DA 80-83, 10-90 USD) - tier 'chợ' Fiverr/Kwork, rủi ro chất lượng thấp; Tier 4 - 'báo hạt giống'/site vệ tinh không tên tuổi - dấu hiệu PBN, KHÔNG nên đưa vào bảng giá Digicom nếu muốn giữ uy tín. Ngành hàng phù hợp: không có dữ liệu trực tiếp trên nguồn đã đọc (không bịa) - suy luận hợp lý: doanh nghiệp xuất khẩu cần uy tín quốc tế, startup gọi vốn nước ngoài cần 'as seen on' cho pitch deck, thương hiệu mở rộng thị trường quốc tế, tài chính-crypto-fintech (ngành RỦI RO, hay bị lạm dụng PR giả/'financial journalist AI-generated puppets'). SEO/GEO/AEO: không có dữ liệu trực tiếp nào nhắc riêng GEO/AEO cho backlink quốc tế - GAP, đối thủ dừng ở khung SEO truyền thống (DA/DR, dofollow), chưa ai định vị theo AI Search/GEO. VAT/hoá đơn: Forbes Việt Nam (đơn vị trong nước, khác dịch vụ booking quốc tế outbound) ghi rõ 'giá không bao gồm VAT'; wire service quốc tế không đề cập VAT (mua qua thẻ tín dụng quốc tế, không có hoá đơn VAT VN chuẩn) - đây là điểm agency VN trung gian mua hộ + xuất hoá đơn VN có lợi thế thật. NGUỒN: seovip.vn, iacdigital.org (2 bài), oriagency.vn, dps.media, miccreative.vn, mona.media, brando.vn, kingnewswire.com, editorial.link, web20ranker.com, linkedin.com (bài phân tích as-seen-on), larslofgren.com, pamperry.substack.com, threads.com (uptopz.com và prglobal.vn lỗi DNS, chưa verify được đầy đủ). ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: session 2026-08-05 14:15
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
+++ b/10-bang-gia-booking/book-bao-tu-khoa-phan-nhom_2026-08-05.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 13/14 nguồn (13 fetch được, 1 lỗi 404), search 'booking báo chí'/'book báo chí'. Loại hình báo: 100% (13/13) chỉ tập trung báo điện tử/báo online; báo giấy/tạp chí chỉ được nhắc như kênh truyền thống, không còn ai bán (2/13); truyền hình VTV/HTV như kênh phụ trợ đa kênh (3/13); phát thanh, OOH, KOL/Influencer chỉ nhắc lướt ở agency đa kênh (1/13). Loại link: chỉ 4/13 nói rõ dofollow/nofollow, 9/13 KHÔNG nhắc loại link - điểm mù lớn của thị trường. Tên đầu báo (xếp theo tần suất, 13 nguồn): VnExpress (7), Kênh14 (5), Dân Trí (5), 24h.com.vn (4), Tuổi Trẻ (4), Zing/ZingNews (4), Eva.vn (3), VietNamNet (3), Soha (2), Thanh Niên (2), CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn (1 lần mỗi báo). Số đầu báo hợp tác đối thủ tự claim: '1000+' (2/13), '300+' (2/13), '200+' (1/13), 'hàng trăm' không con số cụ thể (1/13). Giá: dải rộng không thống nhất đơn vị, phổ biến 200k-15tr/bài (báo lớn ~2tr, tỉnh ~1tr, niche 700k-200k), có nơi phân 3 tier 3tr+/15tr+/35tr+, có nơi phân theo tier 30-150tr/10-30tr/3-10tr; VAT chỉ 1/13 nói rõ 'chưa gồm VAT'; chiết khấu 10-35% theo giá trị HĐ, có agency tới 40%. Quy trình 4-6 bước lặp lại: tư vấn/tiếp nhận yêu cầu -&gt; chọn báo phù hợp -&gt; viết bài (nhiều nơi viết FREE kèm gói) -&gt; ký HĐ/đặt cọc -&gt; đăng -&gt; báo cáo/nghiệm thu; thời gian hoàn thành chỉ 1/13 nêu cụ thể '7-14 ngày'. Ngành hàng phù hợp: bất động sản, ô tô, y tế/sức khoẻ, thời trang, giáo dục, TMĐT, giải trí/gaming/lifestyle, thể thao; ngành CẤM: cờ bạc, nội dung người lớn, lừa đảo (1/13 nêu rõ). Yêu cầu nội dung KHÔNG đồng nhất giữa đối thủ: phổ biến nhất '1000 từ + 5 ảnh, 1-2 link'; có nơi '800-1200 từ, 2-5 ảnh, 1-3 link'; có nơi chỉ '700+ chữ' hoặc '&lt;300 từ' tuỳ báo - GAP: chưa đối thủ nào làm bảng minh bạch chuẩn bài theo TỪNG đầu báo. SEO/backlink: 'backlink dofollow', 'chiến lược SEO hữu hiệu', 'vĩnh viễn không gỡ', 'hỗ trợ thúc đẩy từ khoá', 'tăng top Google' - nhưng 0/13 công bố DR/DA/traffic thật theo từng đầu báo cụ thể. GEO (Generative Engine Optimization)/AEO (Answer Engine Optimization): 0/13 - HOÀN TOÀN không nguồn nào nhắc, kể cả trang cập nhật 2026 - đây là GAP/cơ hội khác biệt lớn nhất thị trường hiện tại. Hành vi/lý do khách hàng cần booking báo: tăng uy tín thương hiệu, xây hình ảnh chuyên nghiệp, tiếp cận khách hàng mục tiêu, hỗ trợ SEO/tìm kiếm, tăng doanh số/chuyển đổi - KHÔNG nguồn nào nhắc cụ thể tình huống 'gọi vốn', 'tuyển dụng', 'xử lý khủng hoảng truyền thông' - GAP hành vi khách hàng chưa ai khai thác. Agency/đối thủ được nhắc làm case tham chiếu: Á Châu Media, Admicro (VCCorp), Life Media (chiết khấu tới 40%), Brandcom (15 năm, khách Vinhomes/FPT), Mona Media; 1 agency sở hữu hệ 7 site riêng để PR chéo (mô hình khác hẳn trung gian đặt bài báo lớn thứ ba). NGUỒN: accesstrade.vn, seovip.vn, itify.vn, bookbaopr.vn, chobao.vn, hapodigital.com, kmedia.vn, tindimedia.vn, songkim.net, nhattinmarketing.com, lennguyenmedia.com, miccreative.vn, tinnghiamedia.vn. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>Báo điện tử, báo giấy, tạp chí, truyền hình, phát thanh, OOH, KOL/Influencer, backlink dofollow, backlink nofollow, DR, DA, traffic, VnExpress, Kênh14, Dân Trí, 24h.com.vn, Tuổi Trẻ, Zing/ZingNews, Eva.vn, VietNamNet, Soha, Thanh Niên, CafeF, Người Lao Động, Báo Giáo Dục, ELLE, Lao Động, Dân Việt, Tiền Phong, TheLEADER, Webtretho, Techz, Thể Thao 247, Thể Thao Văn Hoá, Báo Mới, 2Sao, Tin Tức Online, VOV, Afamily, CafeBiz, GameK, Sức Khỏe &amp; Đời Sống, Batdongsan.com.vn, số đầu báo hợp tác, giá theo bài, VAT, hoá đơn, chiết khấu, quy trình đặt bài, hợp đồng, đặt cọc, nghiệm thu, viết bài PR, số từ, số ảnh, số link, tiêu đề, ngành bất động sản, ngành ô tô, ngành y tế/sức khoẻ, ngành thời trang, ngành giáo dục, ngành TMĐT, ngành giải trí/gaming/lifestyle, ngành thể thao, ngành cấm (cờ bạc, nội dung người lớn, lừa đảo), SEO, entity SEO, guest post, textlink, GEO, AEO, ChatGPT, Gemini, Google AI Overview, xây dựng thương hiệu, uy tín thương hiệu, PR, marketing, agency booking báo, Á Châu Media, Admicro, VCCorp, Life Media, Brandcom, Mona Media.</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1434,7 @@
       <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       <c r="F38" s="5" t="inlineStr"/>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       <c r="F43" s="5" t="inlineStr"/>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       <c r="F44" s="5" t="inlineStr"/>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2033,7 @@
       <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 10 trang cho 4 đầu báo đại diện: VnExpress, Dân Trí, Kênh14, Báo 24h. Loại hình báo: cả 4 đều là báo điện tử có giấy phép báo chí (VnExpress - Bộ KH&amp;CN, Dân Trí - Hội Khuyến học VN, Kênh14/24h - VCCorp/Admicro), KHÔNG phải báo giấy/tạp chí (4/4). Vị trí đăng phân tầng rõ rệt: Top 1/Top ưu tiên trang chủ &gt; Trang chủ Top 3-5 &gt; Chuyên mục nổi bật (Group 1/2) &gt; Tiểu mục/Stream thường (10/10 nguồn). Giá VnExpress: Trang chủ Business/BĐS Top 3-5 = 30-60tr; chuyên mục Sức khỏe/Đời sống/Thể thao = 9-12tr; chuyên mục Du lịch/Công nghệ/Ô tô = 7-10tr; bài tự chuẩn bị nội dung 15-50tr, báo viết hộ +5-10tr; tin ảnh 20-45tr. Giá Dân Trí: khởi điểm 1,8tr, tiểu mục rẻ, Top 1 trang chủ đắt gấp ~8 lần tiểu mục; chèn link mua riêng 500k/link hoặc 3 link/1tr. Giá Kênh14: TOP 1 PC/Mobile 60tr, TOP 1 Mix 90tr, chuyên mục nổi bật (Group 1) 18-20tr, Stream 2 (Group 2) 12tr, Stream 3 8tr, video Type 1 18tr/Type 3 8tr - biên độ toàn dải 4-90tr. Giá Báo 24h: 5-16,6tr/bài theo nhóm chuyên mục và Type 1/Type 2, có nguồn ghi biên hẹp hơn 2-4tr CHƯA VAT - chênh lệch lớn giữa các agency cho cùng 1 báo. VAT/hoá đơn: chỉ 1 nguồn (24h) nêu rõ giá 'chưa gồm 8% VAT', hầu hết nguồn khác không nêu minh bạch. Quy cách bài: tối đa 1.000 từ (10/10 báo); số ảnh khác nhau theo báo - VnExpress 1-3 ảnh không logo/chữ, Dân Trí 6-10 ảnh (tin ảnh tối thiểu 7), Kênh14 tối đa 5 ảnh (tin ảnh 7-10), 24h tối đa 5 ảnh có bản quyền; tiêu đề giới hạn ký tự/từ khác nhau theo báo (VnExpress 13-14 từ, Kênh14/24h tối đa 11 từ, Dân Trí tối đa 75 ký tự); lead/sapo giới hạn (VnExpress 32 từ, Dân Trí 250 ký tự, Kênh14 45 từ, 24h 300 ký tự); thời gian duyệt/đăng 1-4 ngày làm việc tuỳ báo; video Kênh14/Dân Trí tối đa 5 phút, 50MB. Loại link: hầu hết nofollow là mặc định (VnExpress tối đa 2 nofollow, 24h 1 nofollow/bài kèm mua thêm) nhưng có nguồn ghi VnExpress dofollow tối đa 2 link - MÂU THUẪN giữa các agency về loại link cùng 1 báo; không nguồn nào công bố DR/DA theo thang Ahrefs/Moz chuẩn (chỉ 1/10 ước lượng 'DA ~90' không kiểm chứng chéo được). Traffic/pageview: VnExpress ~190 triệu lượt/tháng (organic 60%/direct 27%/social 10%, time-on-page 5,5 phút, bounce 36%); Dân Trí ~120 triệu lượt + 500 triệu pageview/tháng; Kênh14 ~122 triệu pageview + 33,5 triệu visitor/tháng (hoặc 20-30 triệu theo nguồn khác - top 50 website VN); Báo 24h 15-20 triệu lượt/tháng (68% organic) hoặc 180 triệu lượt đọc/tháng theo nguồn khác - chênh lệch số liệu rất lớn giữa các agency cùng nói về 1 báo. Demographic độc giả suy ra ngành hàng phù hợp: VnExpress 25-45 tuổi, thu nhập trung-cao, đô thị lớn -&gt; hợp BĐS, tài chính, giáo dục, du lịch, công nghệ, y tế; Dân Trí độc giả đa dạng sinh viên-doanh nhân -&gt; hợp giáo dục, y tế, ô tô, BĐS, du lịch; Kênh14 độc giả Gen Z/Millennials 18-35 tuổi (64% nữ) -&gt; hợp hàng tiêu dùng, mỹ phẩm/làm đẹp, giải trí, thời trang; Báo 24h độc giả 14-45 tuổi -&gt; hợp BĐS, tài chính-ngân hàng, y tế, làm đẹp, FMCG, giáo dục, du lịch. Mục đích PR/thương hiệu: xây dựng thương hiệu qua 'sức mạnh ngôn từ' (branding qua bài chuẩn báo chí), tăng độ tin cậy nhờ gắn tên tuổi báo lớn - KHÔNG nguồn nào nói rõ mục đích 'ra mắt sản phẩm' cụ thể, chủ yếu định vị chung 'quảng bá thương hiệu'. SEO/backlink: nhấn mạnh nhiều nhất 'bài đăng tồn tại vĩnh viễn, được Google index lâu dài' (4/10, rõ nhất ở 24h). GEO/AEO: KHÔNG nguồn nào trong 10 trang nhắc tới (0/10) - khoảng trống hoàn toàn của thị trường. Hành vi khách hàng chọn đúng đầu báo: theo demographic độc giả khớp ngành/sản phẩm, theo ngân sách (biên độ giá 1,8tr-90tr rất rộng), theo mức uy tín cần có - không nguồn nào có dữ liệu hành vi thật (khảo sát), chỉ suy luận logic. Hình thức bài đặc biệt: photo story/tin ảnh (VnExpress, Dân Trí, Kênh14), video PR (Kênh14, Dân Trí), eMagazine/infographic/interactive (chỉ Dân Trí nhắc tên, không có giá cụ thể). Ràng buộc pháp lý/thủ tục: yêu cầu giấy phép kinh doanh để xác minh trước khi đăng (VnExpress); mục 'Thông tin doanh nghiệp' chỉ tồn tại 2 năm rồi gỡ (1 nguồn); huỷ sau khi đã duyệt bị phạt cố định 2 triệu đồng (1 nguồn). NGUỒN: brando.vn, seodo.vn, miccreative.vn, ecpmedia.vn (bảng giá dạng PDF không đọc được số), marketingai.vn, seovip.vn, prbaochi.com, hapodigital.com. ĐÍNH CHÍNH GEO/AEO (2026-08-05, sau khi user chỉ ra lỗi và verify lại trực tiếp seovip.vn): seovip.vn (nằm trong danh sách nguồn đã đọc) THỰC TẾ CÓ 1 mục riêng 'Tối ưu AI Search AEO/GEO' trong phần lợi ích dịch vụ, nội dung: 'khi thương hiệu được nhắc đến nhiều, có cơ hội xuất hiện trên câu trả lời của ChatGPT, Gemini, Google AI Overview' - agent nghiên cứu ban đầu đã BỎ SÓT mục này. Sửa lại: KHÔNG PHẢI '0 đối thủ nhắc GEO/AEO' - đã có ít nhất 1 đối thủ (seovip.vn) khai thác góc này, nhưng chỉ dừng ở mức nêu tên + 1 câu chung chung, CHƯA giải thích cơ chế cụ thể/cách làm. Cơ hội thật của Digicom là làm SÂU HƠN (giải thích rõ AEO/GEO là gì, cơ chế được AI trích dẫn, cách tối ưu cụ thể cho bài PR/booking báo), không phải 'người đầu tiên nhắc tới' - cần rà lại các trang khác trong danh sách nguồn xem có bỏ sót tương tự không trước khi viết bài dựa vào GAP này.</t>
+          <t>VnExpress, Dân Trí, Kênh14, Báo 24h, báo điện tử, giấy phép báo chí, trang chủ, chuyên mục, box nổi bật, tiểu mục, Top 1, giá theo hạng/vị trí, VAT, hoá đơn, số từ, số ảnh, số link, tiêu đề, lead/sapo, thời gian duyệt bài, thời gian đăng bài, tin ảnh, video PR, eMagazine, infographic, backlink dofollow, backlink nofollow, DR, DA, UR, Ahrefs, traffic, pageview, bounce rate, thời gian trên trang, đối tượng độc giả, demographic, ngành bất động sản, ngành tài chính, ngành giáo dục, ngành y tế, ngành du lịch, ngành công nghệ, ngành mỹ phẩm/làm đẹp, ngành ô tô, ngành hàng tiêu dùng, ngành thời trang, ngành FMCG, xây dựng thương hiệu, uy tín thương hiệu, ra mắt sản phẩm, SEO, index Google, GEO, AEO, ChatGPT, Gemini, Google AI Overview, giấy phép kinh doanh, hợp đồng, phạt huỷ bài.</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2518,7 @@
       <c r="F70" s="8" t="inlineStr"/>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       <c r="F71" s="8" t="inlineStr"/>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
       <c r="F72" s="8" t="inlineStr"/>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
       <c r="F73" s="8" t="inlineStr"/>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       <c r="F74" s="8" t="inlineStr"/>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       <c r="F75" s="8" t="inlineStr"/>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       <c r="F76" s="8" t="inlineStr"/>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       <c r="F77" s="8" t="inlineStr"/>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
       <c r="F78" s="8" t="inlineStr"/>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2727,7 +2727,7 @@
       <c r="F79" s="8" t="inlineStr"/>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2750,7 @@
       <c r="F80" s="8" t="inlineStr"/>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo báo chí đúng chuẩn, không gian phỏng vấn/quay chuyên nghiệp, hồ sơ pháp lý DN, hình ảnh/video/thông tin sản phẩm hỗ trợ. NGUỒN: blog.vn.revu.net, marketingai.vn, oriagency.vn, achau.vn, vietstarmax.vn, trangiadigital.com, vietquangcao.org, mediaz.vn (chỉ đọc được qua snippet, fetch lỗi 403).</t>
+          <t>Banner quảng cáo, TVC, livestream, native ads, advertorial, fanpage, YouTube, TikTok, Instagram, Zalo, group Facebook, báo điện tử, tạp chí, báo giấy, KOL, KOC, Influencer, Nano, Micro, Mid-tier, Macro, Mega, Celeb, Mass Seeder, Engagement Rate, CPM, Reach, Impression, Follower, giá theo bài/post, giá theo giờ, hợp đồng dài hạn, hoa hồng đại lý, chiết khấu, VAT, ngành thời trang/làm đẹp, ngành bất động sản, ngành công nghệ, ngành ẩm thực, ngành du lịch, ngành giáo dục, ngành lifestyle, media booking, media plan, PR, marketing, thương hiệu, thông cáo báo chí, hồ sơ pháp lý doanh nghiệp.</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       <c r="F81" s="8" t="inlineStr"/>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>NGHIÊN CỨU 8 trang (LƯU Ý: dịch vụ này Digicom CHƯA bán, chỉ để tham khảo entity). Loại hình quảng cáo: banner (tĩnh/động, không tìm được số liệu kích thước chuẩn IAB cụ thể trên nguồn nào - không bịa số); PR article/bài PR (tối đa 3 textlink); video commercial/TVC (10-30 giây); livestream (theo giờ, vd 1 giờ = 25 triệu VNĐ); native ads/advertorial; fanpage post (bài mới, share link, reels/video ngắn); OOH (billboard, LED, thang máy, TTTM); phát thanh (khung giờ cố định). Loại hình báo/nền tảng: báo điện tử (Tuổi Trẻ, CafeF, CafeBiz, Dân Trí, Soha, GameK, AutoPro, VTC News, Tiền Phong); tạp chí/báo giấy (kênh truyền thống, chi phí thấp hơn, độc giả trung thành); fanpage Facebook; YouTube; TikTok; Instagram; Zalo; group Facebook (tạo hiệu ứng viral tự nhiên). KOL/KOC/Influencer phân tầng theo follower (số liệu KHÔNG thống nhất giữa các nguồn - cần thận trọng khi trích dẫn): Nano 1K-10K (0,6-6,1 triệu), Micro 10K-50K/100K (5-30,5 triệu), Mid-tier 50K-100K (10-20 triệu), Macro 100K-500K/1M (20-611 triệu), Mega/Celeb 500K-1M+ (50-611 triệu+). Phân loại 3 nhóm: Celeb (nghệ sĩ/đại sứ thương hiệu), Influencer (micro/macro), Mass Seeder (reviewer chuyên ngành hẹp). Ví dụ giá thật tìm được: Trấn Thành 280 triệu, Hoa hậu Kỳ Duyên 200 triệu, Noo Phước Thịnh 150 triệu/bài. Chỉ số đo lường: Engagement Rate = (Like+Comment)/Follower x 100% (ngưỡng tốt &gt;5%); CPM = (Phí booking/Views) x 1.000; Reach; Impression - KHÔNG tìm thấy công thức CPC/CPV/CPL cụ thể trên nguồn đã đọc, không bịa. Giá cả: đơn vị VNĐ/bài, VNĐ/post, VNĐ/giờ (livestream), VNĐ/tháng (hợp đồng dài hạn); hình thức thanh toán KOL: cố định (48,6% phổ biến nhất), theo bậc (28,8%), hoa hồng (19,7%); cam kết 3-6 tháng giảm 20-40%; hoa hồng đại lý chiết khấu 10-35%; KHÔNG nguồn nào nêu rõ VAT/hoá đơn. Ngành hàng theo kênh: thời trang/làm đẹp phù hợp KOL (5-30tr micro, tới 2 tỷ celeb); bất động sản phù hợp KOL (10-30tr micro, 800tr macro); công nghệ phù hợp micro-influencer (8-25tr/bài) và chuyên gia nổi tiếng (150-700tr/bài); ẩm thực/du lịch/giáo dục/lifestyle phù hợp TikTok/Instagram/YouTube. PR/marketing/thương hiệu, media plan: media booking = doanh nghiệp đặt truyền thông trên kênh online (báo điện tử, MXH, KOL) và offline (truyền hình, phát thanh, OOH); agency đóng vai trò trung gian giúp tiết kiệm chi phí; quy trình 4 bước: tư vấn/báo giá -&gt; ký hợp đồng -&gt; biên tập/duyệt nội dung -&gt; khách phê duyệt. Hành vi khách hàng: chọn kênh theo thói quen tiêu thụ media của đối tượng mục tiêu, ngân sách, mức độ nhạy cảm thông tin; cần chuẩn bị thông cáo bá